<commit_message>
update cost-benefits configuration parameters in cb_config_params.xlsx
</commit_message>
<xml_diff>
--- a/ssp_modeling/cost-benefits/cb_config_files/cb_config_params.xlsx
+++ b/ssp_modeling/cost-benefits/cb_config_files/cb_config_params.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10928"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="11130"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/fabianfuentes/git/ssp_mexico/ssp_modeling/cost-benefits/cb_config_files/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/tony/Documents/sisepuede_modeling/ssp_bulgaria/ssp_modeling/cost-benefits/cb_config_files/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7B22CFD6-8403-6446-8AEC-6FA847864C17}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{08F59993-5565-C74E-AD41-546D3286E593}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-40960" yWindow="-5400" windowWidth="30240" windowHeight="18880" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="620" windowWidth="38400" windowHeight="19780" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="tx_table" sheetId="1" r:id="rId1"/>
@@ -17001,7 +17001,7 @@
         <v>462</v>
       </c>
       <c r="C17">
-        <v>300</v>
+        <v>200</v>
       </c>
       <c r="D17" t="s">
         <v>589</v>

</xml_diff>

<commit_message>
fixed wali cost factors
</commit_message>
<xml_diff>
--- a/ssp_modeling/cost-benefits/cb_config_files/cb_config_params.xlsx
+++ b/ssp_modeling/cost-benefits/cb_config_files/cb_config_params.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/tony/Documents/sisepuede_modeling/ssp_bulgaria/ssp_modeling/cost-benefits/cb_config_files/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2C8120B7-BBE4-E045-A741-532229B2D4B1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4EA9959B-E740-1B4B-B783-5192A767FA8E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5920" yWindow="620" windowWidth="27500" windowHeight="19660" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="5920" yWindow="620" windowWidth="27500" windowHeight="19660" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="tx_table" sheetId="1" r:id="rId1"/>
@@ -6296,7 +6296,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="8">
+  <fills count="9">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -6339,6 +6339,12 @@
         <bgColor rgb="FF000000"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -6371,7 +6377,7 @@
       <protection locked="0"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
@@ -6383,6 +6389,7 @@
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="3" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -16573,117 +16580,117 @@
         <v>443</v>
       </c>
     </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A2" t="s">
+    <row r="2" spans="1:12" s="6" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A2" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" s="6" t="s">
         <v>444</v>
       </c>
-      <c r="C2">
+      <c r="C2" s="6">
         <v>-6.5</v>
       </c>
-      <c r="D2" t="s">
+      <c r="D2" s="6" t="s">
         <v>584</v>
       </c>
-      <c r="E2">
-        <v>1</v>
-      </c>
-      <c r="F2" t="s">
+      <c r="E2" s="6">
+        <v>1</v>
+      </c>
+      <c r="F2" s="6" t="s">
         <v>211</v>
       </c>
-      <c r="G2" t="b">
+      <c r="G2" s="6" t="b">
         <v>0</v>
       </c>
-      <c r="H2" t="s">
+      <c r="H2" s="6" t="s">
         <v>598</v>
       </c>
-      <c r="I2" t="s">
+      <c r="I2" s="6" t="s">
         <v>378</v>
       </c>
-      <c r="J2" t="s">
+      <c r="J2" s="6" t="s">
         <v>350</v>
       </c>
-      <c r="K2" t="s">
+      <c r="K2" s="6" t="s">
         <v>687</v>
       </c>
-      <c r="L2" t="s">
+      <c r="L2" s="6" t="s">
         <v>690</v>
       </c>
     </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A3" t="s">
+    <row r="3" spans="1:12" s="6" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A3" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="B3" t="s">
+      <c r="B3" s="6" t="s">
         <v>445</v>
       </c>
-      <c r="C3">
-        <v>-68.099999999999994</v>
-      </c>
-      <c r="D3" t="s">
+      <c r="C3" s="6">
+        <v>-102.1</v>
+      </c>
+      <c r="D3" s="6" t="s">
         <v>584</v>
       </c>
-      <c r="E3">
-        <v>1</v>
-      </c>
-      <c r="F3" t="s">
+      <c r="E3" s="6">
+        <v>1</v>
+      </c>
+      <c r="F3" s="6" t="s">
         <v>212</v>
       </c>
-      <c r="G3" t="b">
+      <c r="G3" s="6" t="b">
         <v>0</v>
       </c>
-      <c r="H3" t="s">
+      <c r="H3" s="6" t="s">
         <v>599</v>
       </c>
-      <c r="I3" t="s">
+      <c r="I3" s="6" t="s">
         <v>378</v>
       </c>
-      <c r="J3" t="s">
+      <c r="J3" s="6" t="s">
         <v>350</v>
       </c>
-      <c r="K3" t="s">
+      <c r="K3" s="6" t="s">
         <v>687</v>
       </c>
-      <c r="L3" t="s">
+      <c r="L3" s="6" t="s">
         <v>690</v>
       </c>
     </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A4" t="s">
+    <row r="4" spans="1:12" s="9" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A4" s="9" t="s">
         <v>7</v>
       </c>
-      <c r="B4" t="s">
+      <c r="B4" s="9" t="s">
         <v>446</v>
       </c>
-      <c r="C4">
-        <v>-102.1</v>
-      </c>
-      <c r="D4" t="s">
+      <c r="C4" s="9">
+        <v>-75.099999999999994</v>
+      </c>
+      <c r="D4" s="9" t="s">
         <v>584</v>
       </c>
-      <c r="E4">
-        <v>1</v>
-      </c>
-      <c r="F4" t="s">
+      <c r="E4" s="9">
+        <v>1</v>
+      </c>
+      <c r="F4" s="9" t="s">
         <v>213</v>
       </c>
-      <c r="G4" t="b">
+      <c r="G4" s="9" t="b">
         <v>0</v>
       </c>
-      <c r="H4" t="s">
+      <c r="H4" s="9" t="s">
         <v>600</v>
       </c>
-      <c r="I4" t="s">
+      <c r="I4" s="9" t="s">
         <v>378</v>
       </c>
-      <c r="J4" t="s">
+      <c r="J4" s="9" t="s">
         <v>350</v>
       </c>
-      <c r="K4" t="s">
+      <c r="K4" s="9" t="s">
         <v>687</v>
       </c>
-      <c r="L4" t="s">
+      <c r="L4" s="9" t="s">
         <v>690</v>
       </c>
     </row>
@@ -16725,79 +16732,79 @@
         <v>690</v>
       </c>
     </row>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A6" t="s">
+    <row r="6" spans="1:12" s="7" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A6" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="B6" t="s">
+      <c r="B6" s="7" t="s">
         <v>448</v>
       </c>
       <c r="C6">
-        <v>-34.1</v>
-      </c>
-      <c r="D6" t="s">
+        <v>-102.1</v>
+      </c>
+      <c r="D6" s="7" t="s">
         <v>584</v>
       </c>
-      <c r="E6">
-        <v>1</v>
-      </c>
-      <c r="F6" t="s">
+      <c r="E6" s="7">
+        <v>1</v>
+      </c>
+      <c r="F6" s="7" t="s">
         <v>215</v>
       </c>
-      <c r="G6" t="b">
+      <c r="G6" s="7" t="b">
         <v>0</v>
       </c>
-      <c r="H6" t="s">
+      <c r="H6" s="7" t="s">
         <v>601</v>
       </c>
-      <c r="I6" t="s">
+      <c r="I6" s="7" t="s">
         <v>378</v>
       </c>
-      <c r="J6" t="s">
+      <c r="J6" s="7" t="s">
         <v>350</v>
       </c>
-      <c r="K6" t="s">
+      <c r="K6" s="7" t="s">
         <v>687</v>
       </c>
-      <c r="L6" t="s">
+      <c r="L6" s="7" t="s">
         <v>690</v>
       </c>
     </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A7" t="s">
+    <row r="7" spans="1:12" s="6" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A7" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="B7" t="s">
+      <c r="B7" s="6" t="s">
         <v>449</v>
       </c>
       <c r="C7">
-        <v>-66.2</v>
-      </c>
-      <c r="D7" t="s">
+        <v>-41.2</v>
+      </c>
+      <c r="D7" s="6" t="s">
         <v>584</v>
       </c>
-      <c r="E7">
-        <v>1</v>
-      </c>
-      <c r="F7" t="s">
+      <c r="E7" s="6">
+        <v>1</v>
+      </c>
+      <c r="F7" s="6" t="s">
         <v>216</v>
       </c>
-      <c r="G7" t="b">
+      <c r="G7" s="6" t="b">
         <v>0</v>
       </c>
-      <c r="H7" t="s">
+      <c r="H7" s="6" t="s">
         <v>602</v>
       </c>
-      <c r="I7" t="s">
+      <c r="I7" s="6" t="s">
         <v>378</v>
       </c>
-      <c r="J7" t="s">
+      <c r="J7" s="6" t="s">
         <v>350</v>
       </c>
-      <c r="K7" t="s">
+      <c r="K7" s="6" t="s">
         <v>687</v>
       </c>
-      <c r="L7" t="s">
+      <c r="L7" s="6" t="s">
         <v>690</v>
       </c>
     </row>

</xml_diff>

<commit_message>
finished tunning cost and benefits and tableau for dave
</commit_message>
<xml_diff>
--- a/ssp_modeling/cost-benefits/cb_config_files/cb_config_params.xlsx
+++ b/ssp_modeling/cost-benefits/cb_config_files/cb_config_params.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/tony/Documents/sisepuede_modeling/ssp_bulgaria/ssp_modeling/cost-benefits/cb_config_files/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FBC5D005-B545-884F-BA1C-4014CF80871F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{35302E24-9C83-754B-8BD7-910CA3A1A3B2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1480" yWindow="660" windowWidth="27500" windowHeight="17660" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="5320" yWindow="5220" windowWidth="27500" windowHeight="17660" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="tx_table" sheetId="1" r:id="rId1"/>
@@ -6296,7 +6296,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="10">
+  <fills count="11">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -6351,6 +6351,12 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF92D050"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -6383,7 +6389,7 @@
       <protection locked="0"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
@@ -6397,8 +6403,7 @@
     <xf numFmtId="0" fontId="3" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -16748,7 +16753,7 @@
       <c r="B6" s="3" t="s">
         <v>448</v>
       </c>
-      <c r="C6" s="12">
+      <c r="C6" s="3">
         <v>-85</v>
       </c>
       <c r="D6" s="3" t="s">
@@ -16779,41 +16784,41 @@
         <v>690</v>
       </c>
     </row>
-    <row r="7" spans="1:12" s="11" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="11" t="s">
+    <row r="7" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A7" t="s">
         <v>10</v>
       </c>
-      <c r="B7" s="11" t="s">
+      <c r="B7" t="s">
         <v>449</v>
       </c>
-      <c r="C7" s="11">
+      <c r="C7">
         <v>-50.2</v>
       </c>
-      <c r="D7" s="11" t="s">
+      <c r="D7" t="s">
         <v>584</v>
       </c>
-      <c r="E7" s="11">
-        <v>1</v>
-      </c>
-      <c r="F7" s="11" t="s">
+      <c r="E7">
+        <v>1</v>
+      </c>
+      <c r="F7" t="s">
         <v>216</v>
       </c>
-      <c r="G7" s="11" t="b">
+      <c r="G7" t="b">
         <v>0</v>
       </c>
-      <c r="H7" s="11" t="s">
+      <c r="H7" t="s">
         <v>602</v>
       </c>
-      <c r="I7" s="11" t="s">
+      <c r="I7" t="s">
         <v>378</v>
       </c>
-      <c r="J7" s="11" t="s">
+      <c r="J7" t="s">
         <v>350</v>
       </c>
-      <c r="K7" s="11" t="s">
+      <c r="K7" t="s">
         <v>687</v>
       </c>
-      <c r="L7" s="11" t="s">
+      <c r="L7" t="s">
         <v>690</v>
       </c>
     </row>
@@ -17121,79 +17126,79 @@
         <v>693</v>
       </c>
     </row>
-    <row r="16" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A16" t="s">
+    <row r="16" spans="1:12" s="11" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A16" s="11" t="s">
         <v>19</v>
       </c>
-      <c r="B16" t="s">
+      <c r="B16" s="11" t="s">
         <v>458</v>
       </c>
-      <c r="C16">
-        <v>500</v>
-      </c>
-      <c r="D16" t="s">
+      <c r="C16" s="11">
+        <v>1000</v>
+      </c>
+      <c r="D16" s="11" t="s">
         <v>586</v>
       </c>
-      <c r="E16">
-        <v>1</v>
-      </c>
-      <c r="F16" t="s">
+      <c r="E16" s="11">
+        <v>1</v>
+      </c>
+      <c r="F16" s="11" t="s">
         <v>225</v>
       </c>
-      <c r="G16" t="b">
+      <c r="G16" s="11" t="b">
         <v>0</v>
       </c>
-      <c r="H16" t="s">
+      <c r="H16" s="11" t="s">
         <v>607</v>
       </c>
-      <c r="I16" t="s">
+      <c r="I16" s="11" t="s">
         <v>383</v>
       </c>
-      <c r="J16" t="s">
+      <c r="J16" s="11" t="s">
         <v>351</v>
       </c>
-      <c r="K16" t="s">
+      <c r="K16" s="11" t="s">
         <v>688</v>
       </c>
-      <c r="L16" t="s">
+      <c r="L16" s="11" t="s">
         <v>694</v>
       </c>
     </row>
-    <row r="17" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A17" t="s">
+    <row r="17" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A17" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="B17" t="s">
+      <c r="B17" s="3" t="s">
         <v>459</v>
       </c>
-      <c r="C17">
-        <v>200</v>
-      </c>
-      <c r="D17" t="s">
+      <c r="C17" s="3">
+        <v>1000</v>
+      </c>
+      <c r="D17" s="3" t="s">
         <v>586</v>
       </c>
-      <c r="E17">
-        <v>1</v>
-      </c>
-      <c r="F17" t="s">
+      <c r="E17" s="3">
+        <v>1</v>
+      </c>
+      <c r="F17" s="3" t="s">
         <v>226</v>
       </c>
-      <c r="G17" t="b">
+      <c r="G17" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="H17" t="s">
+      <c r="H17" s="3" t="s">
         <v>608</v>
       </c>
-      <c r="I17" t="s">
+      <c r="I17" s="3" t="s">
         <v>384</v>
       </c>
-      <c r="J17" t="s">
+      <c r="J17" s="3" t="s">
         <v>351</v>
       </c>
-      <c r="K17" t="s">
+      <c r="K17" s="3" t="s">
         <v>688</v>
       </c>
-      <c r="L17" t="s">
+      <c r="L17" s="3" t="s">
         <v>694</v>
       </c>
     </row>
@@ -18197,497 +18202,497 @@
         <v>699</v>
       </c>
     </row>
-    <row r="44" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A44" t="s">
+    <row r="44" spans="1:12" s="11" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A44" s="11" t="s">
         <v>47</v>
       </c>
-      <c r="B44" s="3" t="s">
+      <c r="B44" s="11" t="s">
         <v>486</v>
       </c>
-      <c r="C44" s="3">
+      <c r="C44" s="11">
         <v>600</v>
       </c>
-      <c r="D44" t="s">
+      <c r="D44" s="11" t="s">
         <v>591</v>
       </c>
-      <c r="E44">
-        <v>1</v>
-      </c>
-      <c r="F44" t="s">
+      <c r="E44" s="11">
+        <v>1</v>
+      </c>
+      <c r="F44" s="11" t="s">
         <v>253</v>
       </c>
-      <c r="G44" t="b">
+      <c r="G44" s="11" t="b">
         <v>0</v>
       </c>
-      <c r="H44" t="s">
+      <c r="H44" s="11" t="s">
         <v>630</v>
       </c>
-      <c r="I44" t="s">
+      <c r="I44" s="11" t="s">
         <v>679</v>
       </c>
-      <c r="J44" t="s">
+      <c r="J44" s="11" t="s">
         <v>353</v>
       </c>
-      <c r="K44" t="s">
+      <c r="K44" s="11" t="s">
         <v>688</v>
       </c>
-      <c r="L44" t="s">
+      <c r="L44" s="11" t="s">
         <v>699</v>
       </c>
     </row>
-    <row r="45" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A45" t="s">
+    <row r="45" spans="1:12" s="11" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A45" s="11" t="s">
         <v>48</v>
       </c>
-      <c r="B45" s="3" t="s">
+      <c r="B45" s="11" t="s">
         <v>487</v>
       </c>
-      <c r="C45" s="3">
+      <c r="C45" s="11">
+        <v>170</v>
+      </c>
+      <c r="D45" s="11" t="s">
+        <v>591</v>
+      </c>
+      <c r="E45" s="11">
+        <v>1</v>
+      </c>
+      <c r="F45" s="11" t="s">
+        <v>254</v>
+      </c>
+      <c r="G45" s="11" t="b">
+        <v>0</v>
+      </c>
+      <c r="H45" s="11" t="s">
+        <v>631</v>
+      </c>
+      <c r="I45" s="11" t="s">
+        <v>679</v>
+      </c>
+      <c r="J45" s="11" t="s">
+        <v>353</v>
+      </c>
+      <c r="K45" s="11" t="s">
+        <v>688</v>
+      </c>
+      <c r="L45" s="11" t="s">
+        <v>699</v>
+      </c>
+    </row>
+    <row r="46" spans="1:12" s="11" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A46" s="11" t="s">
+        <v>49</v>
+      </c>
+      <c r="B46" s="11" t="s">
+        <v>488</v>
+      </c>
+      <c r="C46" s="11">
         <v>285</v>
       </c>
-      <c r="D45" t="s">
+      <c r="D46" s="11" t="s">
         <v>591</v>
       </c>
-      <c r="E45">
-        <v>1</v>
-      </c>
-      <c r="F45" t="s">
-        <v>254</v>
-      </c>
-      <c r="G45" t="b">
+      <c r="E46" s="11">
+        <v>1</v>
+      </c>
+      <c r="F46" s="11" t="s">
+        <v>255</v>
+      </c>
+      <c r="G46" s="11" t="b">
         <v>0</v>
       </c>
-      <c r="H45" t="s">
-        <v>631</v>
-      </c>
-      <c r="I45" t="s">
+      <c r="H46" s="11" t="s">
+        <v>632</v>
+      </c>
+      <c r="I46" s="11" t="s">
         <v>679</v>
       </c>
-      <c r="J45" t="s">
+      <c r="J46" s="11" t="s">
         <v>353</v>
       </c>
-      <c r="K45" t="s">
+      <c r="K46" s="11" t="s">
         <v>688</v>
       </c>
-      <c r="L45" t="s">
+      <c r="L46" s="11" t="s">
         <v>699</v>
       </c>
     </row>
-    <row r="46" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A46" t="s">
-        <v>49</v>
-      </c>
-      <c r="B46" s="3" t="s">
-        <v>488</v>
-      </c>
-      <c r="C46" s="3">
-        <v>285</v>
-      </c>
-      <c r="D46" t="s">
+    <row r="47" spans="1:12" s="11" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A47" s="11" t="s">
+        <v>50</v>
+      </c>
+      <c r="B47" s="11" t="s">
+        <v>489</v>
+      </c>
+      <c r="C47" s="11">
+        <v>300</v>
+      </c>
+      <c r="D47" s="11" t="s">
         <v>591</v>
       </c>
-      <c r="E46">
-        <v>1</v>
-      </c>
-      <c r="F46" t="s">
-        <v>255</v>
-      </c>
-      <c r="G46" t="b">
+      <c r="E47" s="11">
+        <v>1</v>
+      </c>
+      <c r="F47" s="11" t="s">
+        <v>256</v>
+      </c>
+      <c r="G47" s="11" t="b">
         <v>0</v>
       </c>
-      <c r="H46" t="s">
-        <v>632</v>
-      </c>
-      <c r="I46" t="s">
+      <c r="H47" s="11" t="s">
+        <v>633</v>
+      </c>
+      <c r="I47" s="11" t="s">
         <v>679</v>
       </c>
-      <c r="J46" t="s">
+      <c r="J47" s="11" t="s">
         <v>353</v>
       </c>
-      <c r="K46" t="s">
+      <c r="K47" s="11" t="s">
         <v>688</v>
       </c>
-      <c r="L46" t="s">
+      <c r="L47" s="11" t="s">
         <v>699</v>
       </c>
     </row>
-    <row r="47" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A47" t="s">
-        <v>50</v>
-      </c>
-      <c r="B47" s="3" t="s">
-        <v>489</v>
-      </c>
-      <c r="C47" s="3">
+    <row r="48" spans="1:12" s="11" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A48" s="11" t="s">
+        <v>51</v>
+      </c>
+      <c r="B48" s="11" t="s">
+        <v>490</v>
+      </c>
+      <c r="C48" s="11">
         <v>300</v>
       </c>
-      <c r="D47" t="s">
+      <c r="D48" s="11" t="s">
         <v>591</v>
       </c>
-      <c r="E47">
-        <v>1</v>
-      </c>
-      <c r="F47" t="s">
-        <v>256</v>
-      </c>
-      <c r="G47" t="b">
+      <c r="E48" s="11">
+        <v>1</v>
+      </c>
+      <c r="F48" s="11" t="s">
+        <v>257</v>
+      </c>
+      <c r="G48" s="11" t="b">
         <v>0</v>
       </c>
-      <c r="H47" t="s">
-        <v>633</v>
-      </c>
-      <c r="I47" t="s">
+      <c r="H48" s="11" t="s">
+        <v>630</v>
+      </c>
+      <c r="I48" s="11" t="s">
         <v>679</v>
       </c>
-      <c r="J47" t="s">
+      <c r="J48" s="11" t="s">
         <v>353</v>
       </c>
-      <c r="K47" t="s">
+      <c r="K48" s="11" t="s">
         <v>688</v>
       </c>
-      <c r="L47" t="s">
+      <c r="L48" s="11" t="s">
         <v>699</v>
       </c>
     </row>
-    <row r="48" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A48" t="s">
-        <v>51</v>
-      </c>
-      <c r="B48" s="3" t="s">
-        <v>490</v>
-      </c>
-      <c r="C48" s="3">
+    <row r="49" spans="1:12" s="11" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A49" s="11" t="s">
+        <v>52</v>
+      </c>
+      <c r="B49" s="11" t="s">
+        <v>491</v>
+      </c>
+      <c r="C49" s="11">
+        <v>500</v>
+      </c>
+      <c r="D49" s="11" t="s">
+        <v>591</v>
+      </c>
+      <c r="E49" s="11">
+        <v>1</v>
+      </c>
+      <c r="F49" s="11" t="s">
+        <v>258</v>
+      </c>
+      <c r="G49" s="11" t="b">
+        <v>0</v>
+      </c>
+      <c r="H49" s="11" t="s">
+        <v>634</v>
+      </c>
+      <c r="I49" s="11" t="s">
+        <v>679</v>
+      </c>
+      <c r="J49" s="11" t="s">
+        <v>353</v>
+      </c>
+      <c r="K49" s="11" t="s">
+        <v>688</v>
+      </c>
+      <c r="L49" s="11" t="s">
+        <v>699</v>
+      </c>
+    </row>
+    <row r="50" spans="1:12" s="11" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A50" s="11" t="s">
+        <v>53</v>
+      </c>
+      <c r="B50" s="11" t="s">
+        <v>492</v>
+      </c>
+      <c r="C50" s="11">
         <v>300</v>
       </c>
-      <c r="D48" t="s">
+      <c r="D50" s="11" t="s">
         <v>591</v>
       </c>
-      <c r="E48">
-        <v>1</v>
-      </c>
-      <c r="F48" t="s">
-        <v>257</v>
-      </c>
-      <c r="G48" t="b">
+      <c r="E50" s="11">
+        <v>1</v>
+      </c>
+      <c r="F50" s="11" t="s">
+        <v>259</v>
+      </c>
+      <c r="G50" s="11" t="b">
         <v>0</v>
       </c>
-      <c r="H48" t="s">
+      <c r="H50" s="11" t="s">
         <v>630</v>
       </c>
-      <c r="I48" t="s">
+      <c r="I50" s="11" t="s">
         <v>679</v>
       </c>
-      <c r="J48" t="s">
+      <c r="J50" s="11" t="s">
         <v>353</v>
       </c>
-      <c r="K48" t="s">
+      <c r="K50" s="11" t="s">
         <v>688</v>
       </c>
-      <c r="L48" t="s">
+      <c r="L50" s="11" t="s">
         <v>699</v>
       </c>
     </row>
-    <row r="49" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A49" t="s">
-        <v>52</v>
-      </c>
-      <c r="B49" s="3" t="s">
-        <v>491</v>
-      </c>
-      <c r="C49" s="3">
+    <row r="51" spans="1:12" s="11" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A51" s="11" t="s">
+        <v>54</v>
+      </c>
+      <c r="B51" s="11" t="s">
+        <v>493</v>
+      </c>
+      <c r="C51" s="11">
+        <v>400</v>
+      </c>
+      <c r="D51" s="11" t="s">
+        <v>591</v>
+      </c>
+      <c r="E51" s="11">
+        <v>1</v>
+      </c>
+      <c r="F51" s="11" t="s">
+        <v>260</v>
+      </c>
+      <c r="G51" s="11" t="b">
+        <v>0</v>
+      </c>
+      <c r="H51" s="11" t="s">
+        <v>630</v>
+      </c>
+      <c r="I51" s="11" t="s">
+        <v>679</v>
+      </c>
+      <c r="J51" s="11" t="s">
+        <v>353</v>
+      </c>
+      <c r="K51" s="11" t="s">
+        <v>688</v>
+      </c>
+      <c r="L51" s="11" t="s">
+        <v>699</v>
+      </c>
+    </row>
+    <row r="52" spans="1:12" s="11" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A52" s="11" t="s">
+        <v>55</v>
+      </c>
+      <c r="B52" s="11" t="s">
+        <v>494</v>
+      </c>
+      <c r="C52" s="11">
         <v>500</v>
       </c>
-      <c r="D49" t="s">
+      <c r="D52" s="11" t="s">
         <v>591</v>
       </c>
-      <c r="E49">
-        <v>1</v>
-      </c>
-      <c r="F49" t="s">
-        <v>258</v>
-      </c>
-      <c r="G49" t="b">
+      <c r="E52" s="11">
+        <v>1</v>
+      </c>
+      <c r="F52" s="11" t="s">
+        <v>261</v>
+      </c>
+      <c r="G52" s="11" t="b">
         <v>0</v>
       </c>
-      <c r="H49" t="s">
-        <v>634</v>
-      </c>
-      <c r="I49" t="s">
+      <c r="H52" s="11" t="s">
+        <v>635</v>
+      </c>
+      <c r="I52" s="11" t="s">
         <v>679</v>
       </c>
-      <c r="J49" t="s">
+      <c r="J52" s="11" t="s">
         <v>353</v>
       </c>
-      <c r="K49" t="s">
+      <c r="K52" s="11" t="s">
         <v>688</v>
       </c>
-      <c r="L49" t="s">
+      <c r="L52" s="11" t="s">
         <v>699</v>
       </c>
     </row>
-    <row r="50" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A50" t="s">
-        <v>53</v>
-      </c>
-      <c r="B50" s="3" t="s">
-        <v>492</v>
-      </c>
-      <c r="C50" s="3">
+    <row r="53" spans="1:12" s="11" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A53" s="11" t="s">
+        <v>56</v>
+      </c>
+      <c r="B53" s="11" t="s">
+        <v>495</v>
+      </c>
+      <c r="C53" s="11">
         <v>300</v>
       </c>
-      <c r="D50" t="s">
+      <c r="D53" s="11" t="s">
         <v>591</v>
       </c>
-      <c r="E50">
-        <v>1</v>
-      </c>
-      <c r="F50" t="s">
-        <v>259</v>
-      </c>
-      <c r="G50" t="b">
+      <c r="E53" s="11">
+        <v>1</v>
+      </c>
+      <c r="F53" s="11" t="s">
+        <v>262</v>
+      </c>
+      <c r="G53" s="11" t="b">
         <v>0</v>
       </c>
-      <c r="H50" t="s">
-        <v>630</v>
-      </c>
-      <c r="I50" t="s">
+      <c r="H53" s="11" t="s">
+        <v>636</v>
+      </c>
+      <c r="I53" s="11" t="s">
         <v>679</v>
       </c>
-      <c r="J50" t="s">
+      <c r="J53" s="11" t="s">
         <v>353</v>
       </c>
-      <c r="K50" t="s">
+      <c r="K53" s="11" t="s">
         <v>688</v>
       </c>
-      <c r="L50" t="s">
+      <c r="L53" s="11" t="s">
         <v>699</v>
       </c>
     </row>
-    <row r="51" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A51" t="s">
-        <v>54</v>
-      </c>
-      <c r="B51" s="3" t="s">
-        <v>493</v>
-      </c>
-      <c r="C51" s="3">
-        <v>400</v>
-      </c>
-      <c r="D51" t="s">
+    <row r="54" spans="1:12" s="11" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A54" s="11" t="s">
+        <v>57</v>
+      </c>
+      <c r="B54" s="11" t="s">
+        <v>496</v>
+      </c>
+      <c r="C54" s="11">
+        <v>30</v>
+      </c>
+      <c r="D54" s="11" t="s">
         <v>591</v>
       </c>
-      <c r="E51">
-        <v>1</v>
-      </c>
-      <c r="F51" t="s">
-        <v>260</v>
-      </c>
-      <c r="G51" t="b">
+      <c r="E54" s="11">
+        <v>1</v>
+      </c>
+      <c r="F54" s="11" t="s">
+        <v>263</v>
+      </c>
+      <c r="G54" s="11" t="b">
         <v>0</v>
       </c>
-      <c r="H51" t="s">
-        <v>630</v>
-      </c>
-      <c r="I51" t="s">
+      <c r="H54" s="11" t="s">
+        <v>637</v>
+      </c>
+      <c r="I54" s="11" t="s">
         <v>679</v>
       </c>
-      <c r="J51" t="s">
+      <c r="J54" s="11" t="s">
         <v>353</v>
       </c>
-      <c r="K51" t="s">
+      <c r="K54" s="11" t="s">
         <v>688</v>
       </c>
-      <c r="L51" t="s">
+      <c r="L54" s="11" t="s">
         <v>699</v>
       </c>
     </row>
-    <row r="52" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A52" t="s">
-        <v>55</v>
-      </c>
-      <c r="B52" s="3" t="s">
-        <v>494</v>
-      </c>
-      <c r="C52" s="3">
-        <v>500</v>
-      </c>
-      <c r="D52" t="s">
+    <row r="55" spans="1:12" s="11" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A55" s="11" t="s">
+        <v>58</v>
+      </c>
+      <c r="B55" s="11" t="s">
+        <v>497</v>
+      </c>
+      <c r="C55" s="11">
+        <v>300</v>
+      </c>
+      <c r="D55" s="11" t="s">
         <v>591</v>
       </c>
-      <c r="E52">
-        <v>1</v>
-      </c>
-      <c r="F52" t="s">
-        <v>261</v>
-      </c>
-      <c r="G52" t="b">
+      <c r="E55" s="11">
+        <v>1</v>
+      </c>
+      <c r="F55" s="11" t="s">
+        <v>264</v>
+      </c>
+      <c r="G55" s="11" t="b">
         <v>0</v>
       </c>
-      <c r="H52" t="s">
-        <v>635</v>
-      </c>
-      <c r="I52" t="s">
+      <c r="H55" s="11" t="s">
+        <v>638</v>
+      </c>
+      <c r="I55" s="11" t="s">
         <v>679</v>
       </c>
-      <c r="J52" t="s">
+      <c r="J55" s="11" t="s">
         <v>353</v>
       </c>
-      <c r="K52" t="s">
+      <c r="K55" s="11" t="s">
         <v>688</v>
       </c>
-      <c r="L52" t="s">
+      <c r="L55" s="11" t="s">
         <v>699</v>
       </c>
     </row>
-    <row r="53" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A53" t="s">
-        <v>56</v>
-      </c>
-      <c r="B53" s="3" t="s">
-        <v>495</v>
-      </c>
-      <c r="C53" s="3">
+    <row r="56" spans="1:12" s="11" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A56" s="11" t="s">
+        <v>59</v>
+      </c>
+      <c r="B56" s="11" t="s">
+        <v>498</v>
+      </c>
+      <c r="C56" s="11">
         <v>300</v>
       </c>
-      <c r="D53" t="s">
+      <c r="D56" s="11" t="s">
         <v>591</v>
       </c>
-      <c r="E53">
-        <v>1</v>
-      </c>
-      <c r="F53" t="s">
-        <v>262</v>
-      </c>
-      <c r="G53" t="b">
+      <c r="E56" s="11">
+        <v>1</v>
+      </c>
+      <c r="F56" s="11" t="s">
+        <v>265</v>
+      </c>
+      <c r="G56" s="11" t="b">
         <v>0</v>
       </c>
-      <c r="H53" t="s">
-        <v>636</v>
-      </c>
-      <c r="I53" t="s">
+      <c r="H56" s="11" t="s">
+        <v>639</v>
+      </c>
+      <c r="I56" s="11" t="s">
         <v>679</v>
       </c>
-      <c r="J53" t="s">
+      <c r="J56" s="11" t="s">
         <v>353</v>
       </c>
-      <c r="K53" t="s">
+      <c r="K56" s="11" t="s">
         <v>688</v>
       </c>
-      <c r="L53" t="s">
-        <v>699</v>
-      </c>
-    </row>
-    <row r="54" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A54" t="s">
-        <v>57</v>
-      </c>
-      <c r="B54" s="3" t="s">
-        <v>496</v>
-      </c>
-      <c r="C54" s="3">
-        <v>30</v>
-      </c>
-      <c r="D54" t="s">
-        <v>591</v>
-      </c>
-      <c r="E54">
-        <v>1</v>
-      </c>
-      <c r="F54" t="s">
-        <v>263</v>
-      </c>
-      <c r="G54" t="b">
-        <v>0</v>
-      </c>
-      <c r="H54" t="s">
-        <v>637</v>
-      </c>
-      <c r="I54" t="s">
-        <v>679</v>
-      </c>
-      <c r="J54" t="s">
-        <v>353</v>
-      </c>
-      <c r="K54" t="s">
-        <v>688</v>
-      </c>
-      <c r="L54" t="s">
-        <v>699</v>
-      </c>
-    </row>
-    <row r="55" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A55" t="s">
-        <v>58</v>
-      </c>
-      <c r="B55" s="3" t="s">
-        <v>497</v>
-      </c>
-      <c r="C55" s="3">
-        <v>300</v>
-      </c>
-      <c r="D55" t="s">
-        <v>591</v>
-      </c>
-      <c r="E55">
-        <v>1</v>
-      </c>
-      <c r="F55" t="s">
-        <v>264</v>
-      </c>
-      <c r="G55" t="b">
-        <v>0</v>
-      </c>
-      <c r="H55" t="s">
-        <v>638</v>
-      </c>
-      <c r="I55" t="s">
-        <v>679</v>
-      </c>
-      <c r="J55" t="s">
-        <v>353</v>
-      </c>
-      <c r="K55" t="s">
-        <v>688</v>
-      </c>
-      <c r="L55" t="s">
-        <v>699</v>
-      </c>
-    </row>
-    <row r="56" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A56" t="s">
-        <v>59</v>
-      </c>
-      <c r="B56" s="3" t="s">
-        <v>498</v>
-      </c>
-      <c r="C56" s="3">
-        <v>300</v>
-      </c>
-      <c r="D56" t="s">
-        <v>591</v>
-      </c>
-      <c r="E56">
-        <v>1</v>
-      </c>
-      <c r="F56" t="s">
-        <v>265</v>
-      </c>
-      <c r="G56" t="b">
-        <v>0</v>
-      </c>
-      <c r="H56" t="s">
-        <v>639</v>
-      </c>
-      <c r="I56" t="s">
-        <v>679</v>
-      </c>
-      <c r="J56" t="s">
-        <v>353</v>
-      </c>
-      <c r="K56" t="s">
-        <v>688</v>
-      </c>
-      <c r="L56" t="s">
+      <c r="L56" s="11" t="s">
         <v>699</v>
       </c>
     </row>

</xml_diff>

<commit_message>
upload latest code for cost and benefits
</commit_message>
<xml_diff>
--- a/ssp_modeling/cost-benefits/cb_config_files/cb_config_params.xlsx
+++ b/ssp_modeling/cost-benefits/cb_config_files/cb_config_params.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/tony/Documents/sisepuede_modeling/ssp_bulgaria/ssp_modeling/cost-benefits/cb_config_files/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{35302E24-9C83-754B-8BD7-910CA3A1A3B2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A3E9351C-F3B4-3749-803C-68AFD0313160}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5320" yWindow="5220" windowWidth="27500" windowHeight="17660" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="29100" yWindow="7000" windowWidth="27720" windowHeight="17980" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="tx_table" sheetId="1" r:id="rId1"/>
@@ -6296,7 +6296,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="11">
+  <fills count="12">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -6312,12 +6312,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="6" tint="0.59999389629810485"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="3" tint="0.79998168889431442"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -6357,6 +6351,18 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.39997558519241921"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -6389,7 +6395,7 @@
       <protection locked="0"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
@@ -6399,11 +6405,13 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -9830,20 +9838,20 @@
         <v>435</v>
       </c>
     </row>
-    <row r="184" spans="1:5" s="7" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A184" s="7" t="s">
+    <row r="184" spans="1:5" s="6" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A184" s="6" t="s">
         <v>2046</v>
       </c>
-      <c r="B184" s="7" t="s">
+      <c r="B184" s="6" t="s">
         <v>329</v>
       </c>
-      <c r="C184" s="7" t="s">
+      <c r="C184" s="6" t="s">
         <v>376</v>
       </c>
-      <c r="D184" s="7" t="s">
+      <c r="D184" s="6" t="s">
         <v>417</v>
       </c>
-      <c r="E184" s="7" t="s">
+      <c r="E184" s="6" t="s">
         <v>435</v>
       </c>
     </row>
@@ -10255,82 +10263,82 @@
         <v>435</v>
       </c>
     </row>
-    <row r="209" spans="1:5" s="7" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A209" s="7" t="s">
+    <row r="209" spans="1:5" s="6" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A209" s="6" t="s">
         <v>2038</v>
       </c>
-      <c r="B209" s="7" t="s">
+      <c r="B209" s="6" t="s">
         <v>2043</v>
       </c>
-      <c r="C209" s="7" t="s">
+      <c r="C209" s="6" t="s">
         <v>351</v>
       </c>
-      <c r="D209" s="7" t="s">
+      <c r="D209" s="6" t="s">
         <v>433</v>
       </c>
-      <c r="E209" s="7" t="s">
+      <c r="E209" s="6" t="s">
         <v>435</v>
       </c>
     </row>
-    <row r="210" spans="1:5" s="7" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A210" s="7" t="s">
+    <row r="210" spans="1:5" s="6" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A210" s="6" t="s">
         <v>2039</v>
       </c>
-      <c r="B210" s="7" t="s">
+      <c r="B210" s="6" t="s">
         <v>2044</v>
       </c>
-      <c r="C210" s="7" t="s">
+      <c r="C210" s="6" t="s">
         <v>351</v>
       </c>
-      <c r="D210" s="7" t="s">
+      <c r="D210" s="6" t="s">
         <v>433</v>
       </c>
-      <c r="E210" s="7" t="s">
+      <c r="E210" s="6" t="s">
         <v>435</v>
       </c>
     </row>
-    <row r="211" spans="1:5" s="7" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A211" s="7" t="s">
+    <row r="211" spans="1:5" s="6" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A211" s="6" t="s">
         <v>2040</v>
       </c>
-      <c r="B211" s="7" t="s">
+      <c r="B211" s="6" t="s">
         <v>2045</v>
       </c>
-      <c r="C211" s="7" t="s">
+      <c r="C211" s="6" t="s">
         <v>351</v>
       </c>
-      <c r="D211" s="7" t="s">
+      <c r="D211" s="6" t="s">
         <v>433</v>
       </c>
-      <c r="E211" s="7" t="s">
+      <c r="E211" s="6" t="s">
         <v>435</v>
       </c>
     </row>
     <row r="212" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A212" s="8" t="s">
+      <c r="A212" s="7" t="s">
         <v>2049</v>
       </c>
-      <c r="B212" s="7" t="s">
+      <c r="B212" s="6" t="s">
         <v>2054</v>
       </c>
-      <c r="C212" s="7" t="s">
+      <c r="C212" s="6" t="s">
         <v>2056</v>
       </c>
-      <c r="E212" s="7" t="s">
+      <c r="E212" s="6" t="s">
         <v>435</v>
       </c>
     </row>
     <row r="213" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A213" s="8" t="s">
+      <c r="A213" s="7" t="s">
         <v>2050</v>
       </c>
-      <c r="B213" s="7" t="s">
+      <c r="B213" s="6" t="s">
         <v>2055</v>
       </c>
-      <c r="C213" s="7" t="s">
+      <c r="C213" s="6" t="s">
         <v>2056</v>
       </c>
-      <c r="E213" s="7" t="s">
+      <c r="E213" s="6" t="s">
         <v>435</v>
       </c>
     </row>
@@ -16594,193 +16602,193 @@
         <v>443</v>
       </c>
     </row>
-    <row r="2" spans="1:12" s="9" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="9" t="s">
+    <row r="2" spans="1:12" s="8" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A2" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="B2" s="9" t="s">
+      <c r="B2" s="8" t="s">
         <v>444</v>
       </c>
-      <c r="C2" s="9">
+      <c r="C2" s="8">
         <v>-6.5</v>
       </c>
-      <c r="D2" s="9" t="s">
+      <c r="D2" s="8" t="s">
         <v>584</v>
       </c>
-      <c r="E2" s="9">
-        <v>1</v>
-      </c>
-      <c r="F2" s="9" t="s">
+      <c r="E2" s="8">
+        <v>1</v>
+      </c>
+      <c r="F2" s="8" t="s">
         <v>211</v>
       </c>
-      <c r="G2" s="9" t="b">
+      <c r="G2" s="8" t="b">
         <v>0</v>
       </c>
-      <c r="H2" s="9" t="s">
+      <c r="H2" s="8" t="s">
         <v>598</v>
       </c>
-      <c r="I2" s="9" t="s">
+      <c r="I2" s="8" t="s">
         <v>378</v>
       </c>
-      <c r="J2" s="9" t="s">
+      <c r="J2" s="8" t="s">
         <v>350</v>
       </c>
-      <c r="K2" s="9" t="s">
+      <c r="K2" s="8" t="s">
         <v>687</v>
       </c>
-      <c r="L2" s="9" t="s">
+      <c r="L2" s="8" t="s">
         <v>690</v>
       </c>
     </row>
-    <row r="3" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="3" t="s">
+    <row r="3" spans="1:12" s="11" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A3" s="11" t="s">
         <v>6</v>
       </c>
-      <c r="B3" s="3" t="s">
+      <c r="B3" s="11" t="s">
         <v>445</v>
       </c>
-      <c r="C3" s="3">
-        <v>-88</v>
-      </c>
-      <c r="D3" s="3" t="s">
+      <c r="C3" s="11">
+        <v>-200</v>
+      </c>
+      <c r="D3" s="11" t="s">
         <v>584</v>
       </c>
-      <c r="E3" s="3">
-        <v>1</v>
-      </c>
-      <c r="F3" s="3" t="s">
+      <c r="E3" s="11">
+        <v>1</v>
+      </c>
+      <c r="F3" s="11" t="s">
         <v>212</v>
       </c>
-      <c r="G3" s="3" t="b">
+      <c r="G3" s="11" t="b">
         <v>0</v>
       </c>
-      <c r="H3" s="3" t="s">
+      <c r="H3" s="11" t="s">
         <v>599</v>
       </c>
-      <c r="I3" s="3" t="s">
+      <c r="I3" s="11" t="s">
         <v>378</v>
       </c>
-      <c r="J3" s="3" t="s">
+      <c r="J3" s="11" t="s">
         <v>350</v>
       </c>
-      <c r="K3" s="3" t="s">
+      <c r="K3" s="11" t="s">
         <v>687</v>
       </c>
-      <c r="L3" s="3" t="s">
+      <c r="L3" s="11" t="s">
         <v>690</v>
       </c>
     </row>
-    <row r="4" spans="1:12" s="9" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="9" t="s">
+    <row r="4" spans="1:12" s="11" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A4" s="11" t="s">
         <v>7</v>
       </c>
-      <c r="B4" s="9" t="s">
+      <c r="B4" s="11" t="s">
         <v>446</v>
       </c>
-      <c r="C4" s="9">
-        <v>-50</v>
-      </c>
-      <c r="D4" s="9" t="s">
+      <c r="C4" s="11">
+        <v>-180</v>
+      </c>
+      <c r="D4" s="11" t="s">
         <v>584</v>
       </c>
-      <c r="E4" s="9">
-        <v>1</v>
-      </c>
-      <c r="F4" s="9" t="s">
+      <c r="E4" s="11">
+        <v>1</v>
+      </c>
+      <c r="F4" s="11" t="s">
         <v>213</v>
       </c>
-      <c r="G4" s="9" t="b">
+      <c r="G4" s="11" t="b">
         <v>0</v>
       </c>
-      <c r="H4" s="9" t="s">
+      <c r="H4" s="11" t="s">
         <v>600</v>
       </c>
-      <c r="I4" s="9" t="s">
+      <c r="I4" s="11" t="s">
         <v>378</v>
       </c>
-      <c r="J4" s="9" t="s">
+      <c r="J4" s="11" t="s">
         <v>350</v>
       </c>
-      <c r="K4" s="9" t="s">
+      <c r="K4" s="11" t="s">
         <v>687</v>
       </c>
-      <c r="L4" s="9" t="s">
+      <c r="L4" s="11" t="s">
         <v>690</v>
       </c>
     </row>
-    <row r="5" spans="1:12" s="9" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="9" t="s">
+    <row r="5" spans="1:12" s="8" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A5" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="B5" s="9" t="s">
+      <c r="B5" s="8" t="s">
         <v>447</v>
       </c>
-      <c r="C5" s="9">
+      <c r="C5" s="8">
         <v>-6.5</v>
       </c>
-      <c r="D5" s="9" t="s">
+      <c r="D5" s="8" t="s">
         <v>584</v>
       </c>
-      <c r="E5" s="9">
-        <v>1</v>
-      </c>
-      <c r="F5" s="9" t="s">
+      <c r="E5" s="8">
+        <v>1</v>
+      </c>
+      <c r="F5" s="8" t="s">
         <v>214</v>
       </c>
-      <c r="G5" s="9" t="b">
+      <c r="G5" s="8" t="b">
         <v>0</v>
       </c>
-      <c r="H5" s="9" t="s">
+      <c r="H5" s="8" t="s">
         <v>598</v>
       </c>
-      <c r="I5" s="9" t="s">
+      <c r="I5" s="8" t="s">
         <v>378</v>
       </c>
-      <c r="J5" s="9" t="s">
+      <c r="J5" s="8" t="s">
         <v>350</v>
       </c>
-      <c r="K5" s="9" t="s">
+      <c r="K5" s="8" t="s">
         <v>687</v>
       </c>
-      <c r="L5" s="9" t="s">
+      <c r="L5" s="8" t="s">
         <v>690</v>
       </c>
     </row>
-    <row r="6" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="3" t="s">
+    <row r="6" spans="1:12" s="12" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A6" s="12" t="s">
         <v>9</v>
       </c>
-      <c r="B6" s="3" t="s">
+      <c r="B6" s="12" t="s">
         <v>448</v>
       </c>
-      <c r="C6" s="3">
-        <v>-85</v>
-      </c>
-      <c r="D6" s="3" t="s">
+      <c r="C6" s="12">
+        <v>-90</v>
+      </c>
+      <c r="D6" s="12" t="s">
         <v>584</v>
       </c>
-      <c r="E6" s="3">
-        <v>1</v>
-      </c>
-      <c r="F6" s="3" t="s">
+      <c r="E6" s="12">
+        <v>1</v>
+      </c>
+      <c r="F6" s="12" t="s">
         <v>215</v>
       </c>
-      <c r="G6" s="3" t="b">
+      <c r="G6" s="12" t="b">
         <v>0</v>
       </c>
-      <c r="H6" s="3" t="s">
+      <c r="H6" s="12" t="s">
         <v>601</v>
       </c>
-      <c r="I6" s="3" t="s">
+      <c r="I6" s="12" t="s">
         <v>378</v>
       </c>
-      <c r="J6" s="3" t="s">
+      <c r="J6" s="12" t="s">
         <v>350</v>
       </c>
-      <c r="K6" s="3" t="s">
+      <c r="K6" s="12" t="s">
         <v>687</v>
       </c>
-      <c r="L6" s="3" t="s">
+      <c r="L6" s="12" t="s">
         <v>690</v>
       </c>
     </row>
@@ -17126,41 +17134,41 @@
         <v>693</v>
       </c>
     </row>
-    <row r="16" spans="1:12" s="11" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A16" s="11" t="s">
+    <row r="16" spans="1:12" s="10" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A16" s="10" t="s">
         <v>19</v>
       </c>
-      <c r="B16" s="11" t="s">
+      <c r="B16" s="10" t="s">
         <v>458</v>
       </c>
-      <c r="C16" s="11">
+      <c r="C16" s="10">
         <v>1000</v>
       </c>
-      <c r="D16" s="11" t="s">
+      <c r="D16" s="10" t="s">
         <v>586</v>
       </c>
-      <c r="E16" s="11">
-        <v>1</v>
-      </c>
-      <c r="F16" s="11" t="s">
+      <c r="E16" s="10">
+        <v>1</v>
+      </c>
+      <c r="F16" s="10" t="s">
         <v>225</v>
       </c>
-      <c r="G16" s="11" t="b">
+      <c r="G16" s="10" t="b">
         <v>0</v>
       </c>
-      <c r="H16" s="11" t="s">
+      <c r="H16" s="10" t="s">
         <v>607</v>
       </c>
-      <c r="I16" s="11" t="s">
+      <c r="I16" s="10" t="s">
         <v>383</v>
       </c>
-      <c r="J16" s="11" t="s">
+      <c r="J16" s="10" t="s">
         <v>351</v>
       </c>
-      <c r="K16" s="11" t="s">
+      <c r="K16" s="10" t="s">
         <v>688</v>
       </c>
-      <c r="L16" s="11" t="s">
+      <c r="L16" s="10" t="s">
         <v>694</v>
       </c>
     </row>
@@ -17354,159 +17362,159 @@
         <v>695</v>
       </c>
     </row>
-    <row r="22" spans="1:12" s="7" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A22" s="7" t="s">
+    <row r="22" spans="1:12" s="6" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A22" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="B22" s="7" t="s">
+      <c r="B22" s="6" t="s">
         <v>464</v>
       </c>
-      <c r="C22" s="7">
+      <c r="C22" s="6">
         <f>-18</f>
         <v>-18</v>
       </c>
-      <c r="D22" s="7" t="s">
+      <c r="D22" s="6" t="s">
         <v>588</v>
       </c>
-      <c r="E22" s="7">
-        <v>1</v>
-      </c>
-      <c r="F22" s="7" t="s">
+      <c r="E22" s="6">
+        <v>1</v>
+      </c>
+      <c r="F22" s="6" t="s">
         <v>231</v>
       </c>
-      <c r="G22" s="7" t="b">
-        <v>1</v>
-      </c>
-      <c r="H22" s="7" t="s">
+      <c r="G22" s="6" t="b">
+        <v>1</v>
+      </c>
+      <c r="H22" s="6" t="s">
         <v>613</v>
       </c>
-      <c r="I22" s="7" t="s">
+      <c r="I22" s="6" t="s">
         <v>678</v>
       </c>
-      <c r="J22" s="7" t="s">
+      <c r="J22" s="6" t="s">
         <v>350</v>
       </c>
-      <c r="K22" s="7" t="s">
+      <c r="K22" s="6" t="s">
         <v>688</v>
       </c>
-      <c r="L22" s="7" t="s">
+      <c r="L22" s="6" t="s">
         <v>696</v>
       </c>
     </row>
-    <row r="23" spans="1:12" s="6" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A23" s="6" t="s">
+    <row r="23" spans="1:12" s="5" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A23" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="B23" s="6" t="s">
+      <c r="B23" s="5" t="s">
         <v>465</v>
       </c>
-      <c r="C23" s="6">
+      <c r="C23" s="5">
         <f>-18</f>
         <v>-18</v>
       </c>
-      <c r="D23" s="6" t="s">
+      <c r="D23" s="5" t="s">
         <v>588</v>
       </c>
-      <c r="E23" s="6">
-        <v>1</v>
-      </c>
-      <c r="F23" s="6" t="s">
+      <c r="E23" s="5">
+        <v>1</v>
+      </c>
+      <c r="F23" s="5" t="s">
         <v>232</v>
       </c>
-      <c r="G23" s="6" t="b">
-        <v>1</v>
-      </c>
-      <c r="H23" s="6" t="s">
+      <c r="G23" s="5" t="b">
+        <v>1</v>
+      </c>
+      <c r="H23" s="5" t="s">
         <v>614</v>
       </c>
-      <c r="I23" s="6" t="s">
+      <c r="I23" s="5" t="s">
         <v>678</v>
       </c>
-      <c r="J23" s="6" t="s">
+      <c r="J23" s="5" t="s">
         <v>350</v>
       </c>
-      <c r="K23" s="6" t="s">
+      <c r="K23" s="5" t="s">
         <v>688</v>
       </c>
-      <c r="L23" s="6" t="s">
+      <c r="L23" s="5" t="s">
         <v>696</v>
       </c>
     </row>
-    <row r="24" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A24" s="4" t="s">
+    <row r="24" spans="1:12" s="11" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A24" s="11" t="s">
         <v>27</v>
       </c>
-      <c r="B24" s="4" t="s">
+      <c r="B24" s="11" t="s">
         <v>466</v>
       </c>
-      <c r="C24" s="4">
-        <f>-70/3</f>
-        <v>-23.333333333333332</v>
-      </c>
-      <c r="D24" t="s">
+      <c r="C24" s="11">
+        <f>-70/2</f>
+        <v>-35</v>
+      </c>
+      <c r="D24" s="11" t="s">
         <v>588</v>
       </c>
-      <c r="E24">
-        <v>1</v>
-      </c>
-      <c r="F24" t="s">
+      <c r="E24" s="11">
+        <v>1</v>
+      </c>
+      <c r="F24" s="11" t="s">
         <v>233</v>
       </c>
-      <c r="G24" t="b">
-        <v>1</v>
-      </c>
-      <c r="H24" t="s">
+      <c r="G24" s="11" t="b">
+        <v>1</v>
+      </c>
+      <c r="H24" s="11" t="s">
         <v>615</v>
       </c>
-      <c r="I24" t="s">
+      <c r="I24" s="11" t="s">
         <v>678</v>
       </c>
-      <c r="J24" t="s">
+      <c r="J24" s="11" t="s">
         <v>350</v>
       </c>
-      <c r="K24" t="s">
+      <c r="K24" s="11" t="s">
         <v>688</v>
       </c>
-      <c r="L24" t="s">
+      <c r="L24" s="11" t="s">
         <v>696</v>
       </c>
     </row>
-    <row r="25" spans="1:12" s="6" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A25" s="6" t="s">
+    <row r="25" spans="1:12" s="11" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A25" s="11" t="s">
         <v>28</v>
       </c>
-      <c r="B25" s="6" t="s">
+      <c r="B25" s="11" t="s">
         <v>467</v>
       </c>
-      <c r="C25" s="6">
-        <f>-3.2</f>
-        <v>-3.2</v>
-      </c>
-      <c r="D25" s="6" t="s">
+      <c r="C25" s="11">
+        <f>-8</f>
+        <v>-8</v>
+      </c>
+      <c r="D25" s="11" t="s">
         <v>588</v>
       </c>
-      <c r="E25" s="6">
-        <v>1</v>
-      </c>
-      <c r="F25" s="6" t="s">
+      <c r="E25" s="11">
+        <v>1</v>
+      </c>
+      <c r="F25" s="11" t="s">
         <v>234</v>
       </c>
-      <c r="G25" s="6" t="b">
-        <v>1</v>
-      </c>
-      <c r="H25" s="6" t="s">
+      <c r="G25" s="11" t="b">
+        <v>1</v>
+      </c>
+      <c r="H25" s="11" t="s">
         <v>616</v>
       </c>
-      <c r="I25" s="6" t="s">
+      <c r="I25" s="11" t="s">
         <v>678</v>
       </c>
-      <c r="J25" s="6" t="s">
+      <c r="J25" s="11" t="s">
         <v>350</v>
       </c>
-      <c r="K25" s="6" t="s">
+      <c r="K25" s="11" t="s">
         <v>688</v>
       </c>
-      <c r="L25" s="6" t="s">
+      <c r="L25" s="11" t="s">
         <v>696</v>
       </c>
     </row>
@@ -17549,276 +17557,276 @@
         <v>696</v>
       </c>
     </row>
-    <row r="27" spans="1:12" s="6" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A27" s="6" t="s">
+    <row r="27" spans="1:12" s="11" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A27" s="11" t="s">
         <v>30</v>
       </c>
-      <c r="B27" s="6" t="s">
+      <c r="B27" s="11" t="s">
         <v>469</v>
       </c>
-      <c r="C27" s="6">
-        <f>-13</f>
-        <v>-13</v>
-      </c>
-      <c r="D27" s="6" t="s">
+      <c r="C27" s="11">
+        <f>-15</f>
+        <v>-15</v>
+      </c>
+      <c r="D27" s="11" t="s">
         <v>588</v>
       </c>
-      <c r="E27" s="6">
-        <v>1</v>
-      </c>
-      <c r="F27" s="6" t="s">
+      <c r="E27" s="11">
+        <v>1</v>
+      </c>
+      <c r="F27" s="11" t="s">
         <v>236</v>
       </c>
-      <c r="G27" s="6" t="b">
-        <v>1</v>
-      </c>
-      <c r="H27" s="6" t="s">
+      <c r="G27" s="11" t="b">
+        <v>1</v>
+      </c>
+      <c r="H27" s="11" t="s">
         <v>618</v>
       </c>
-      <c r="I27" s="6" t="s">
+      <c r="I27" s="11" t="s">
         <v>678</v>
       </c>
-      <c r="J27" s="6" t="s">
+      <c r="J27" s="11" t="s">
         <v>350</v>
       </c>
-      <c r="K27" s="6" t="s">
+      <c r="K27" s="11" t="s">
         <v>688</v>
       </c>
-      <c r="L27" s="6" t="s">
+      <c r="L27" s="11" t="s">
         <v>696</v>
       </c>
     </row>
-    <row r="28" spans="1:12" s="9" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A28" s="9" t="s">
+    <row r="28" spans="1:12" s="11" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A28" s="11" t="s">
         <v>31</v>
       </c>
-      <c r="B28" s="9" t="s">
+      <c r="B28" s="11" t="s">
         <v>470</v>
       </c>
-      <c r="C28" s="9">
-        <f>-0.0001</f>
-        <v>-1E-4</v>
-      </c>
-      <c r="D28" s="9" t="s">
+      <c r="C28" s="11">
+        <f>-0.2</f>
+        <v>-0.2</v>
+      </c>
+      <c r="D28" s="11" t="s">
         <v>589</v>
       </c>
-      <c r="E28" s="9">
-        <v>1</v>
-      </c>
-      <c r="F28" s="9" t="s">
+      <c r="E28" s="11">
+        <v>1</v>
+      </c>
+      <c r="F28" s="11" t="s">
         <v>237</v>
       </c>
-      <c r="G28" s="9" t="b">
+      <c r="G28" s="11" t="b">
         <v>0</v>
       </c>
-      <c r="H28" s="9" t="s">
+      <c r="H28" s="11" t="s">
         <v>619</v>
       </c>
-      <c r="I28" s="9" t="s">
+      <c r="I28" s="11" t="s">
         <v>387</v>
       </c>
-      <c r="J28" s="9" t="s">
+      <c r="J28" s="11" t="s">
         <v>352</v>
       </c>
-      <c r="K28" s="9" t="s">
+      <c r="K28" s="11" t="s">
         <v>688</v>
       </c>
-      <c r="L28" s="9" t="s">
+      <c r="L28" s="11" t="s">
         <v>697</v>
       </c>
     </row>
-    <row r="29" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A29" s="3" t="s">
+    <row r="29" spans="1:12" s="11" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A29" s="11" t="s">
         <v>32</v>
       </c>
-      <c r="B29" s="3" t="s">
+      <c r="B29" s="11" t="s">
         <v>471</v>
       </c>
-      <c r="C29" s="3">
-        <f t="shared" ref="C29:C33" si="0">-0.0001</f>
-        <v>-1E-4</v>
-      </c>
-      <c r="D29" s="3" t="s">
+      <c r="C29" s="11">
+        <f t="shared" ref="C29:C33" si="0">-0.2</f>
+        <v>-0.2</v>
+      </c>
+      <c r="D29" s="11" t="s">
         <v>589</v>
       </c>
-      <c r="E29" s="3">
-        <v>1</v>
-      </c>
-      <c r="F29" s="3" t="s">
+      <c r="E29" s="11">
+        <v>1</v>
+      </c>
+      <c r="F29" s="11" t="s">
         <v>238</v>
       </c>
-      <c r="G29" s="3" t="b">
+      <c r="G29" s="11" t="b">
         <v>0</v>
       </c>
-      <c r="H29" s="3" t="s">
+      <c r="H29" s="11" t="s">
         <v>620</v>
       </c>
-      <c r="I29" s="3" t="s">
+      <c r="I29" s="11" t="s">
         <v>387</v>
       </c>
-      <c r="J29" s="3" t="s">
+      <c r="J29" s="11" t="s">
         <v>352</v>
       </c>
-      <c r="K29" s="3" t="s">
+      <c r="K29" s="11" t="s">
         <v>688</v>
       </c>
-      <c r="L29" s="3" t="s">
+      <c r="L29" s="11" t="s">
         <v>697</v>
       </c>
     </row>
-    <row r="30" spans="1:12" s="9" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A30" s="9" t="s">
+    <row r="30" spans="1:12" s="11" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A30" s="11" t="s">
         <v>33</v>
       </c>
-      <c r="B30" s="9" t="s">
+      <c r="B30" s="11" t="s">
         <v>472</v>
       </c>
-      <c r="C30" s="9">
+      <c r="C30" s="11">
         <f t="shared" si="0"/>
-        <v>-1E-4</v>
-      </c>
-      <c r="D30" s="9" t="s">
+        <v>-0.2</v>
+      </c>
+      <c r="D30" s="11" t="s">
         <v>589</v>
       </c>
-      <c r="E30" s="9">
-        <v>1</v>
-      </c>
-      <c r="F30" s="9" t="s">
+      <c r="E30" s="11">
+        <v>1</v>
+      </c>
+      <c r="F30" s="11" t="s">
         <v>239</v>
       </c>
-      <c r="G30" s="9" t="b">
+      <c r="G30" s="11" t="b">
         <v>0</v>
       </c>
-      <c r="H30" s="9" t="s">
+      <c r="H30" s="11" t="s">
         <v>621</v>
       </c>
-      <c r="I30" s="9" t="s">
+      <c r="I30" s="11" t="s">
         <v>387</v>
       </c>
-      <c r="J30" s="9" t="s">
+      <c r="J30" s="11" t="s">
         <v>352</v>
       </c>
-      <c r="K30" s="9" t="s">
+      <c r="K30" s="11" t="s">
         <v>688</v>
       </c>
-      <c r="L30" s="9" t="s">
+      <c r="L30" s="11" t="s">
         <v>697</v>
       </c>
     </row>
-    <row r="31" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A31" s="3" t="s">
+    <row r="31" spans="1:12" s="11" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A31" s="11" t="s">
         <v>34</v>
       </c>
-      <c r="B31" s="3" t="s">
+      <c r="B31" s="11" t="s">
         <v>473</v>
       </c>
-      <c r="C31" s="3">
+      <c r="C31" s="11">
         <f t="shared" si="0"/>
-        <v>-1E-4</v>
-      </c>
-      <c r="D31" s="3" t="s">
+        <v>-0.2</v>
+      </c>
+      <c r="D31" s="11" t="s">
         <v>589</v>
       </c>
-      <c r="E31" s="3">
-        <v>1</v>
-      </c>
-      <c r="F31" s="3" t="s">
+      <c r="E31" s="11">
+        <v>1</v>
+      </c>
+      <c r="F31" s="11" t="s">
         <v>240</v>
       </c>
-      <c r="G31" s="3" t="b">
+      <c r="G31" s="11" t="b">
         <v>0</v>
       </c>
-      <c r="H31" s="3" t="s">
+      <c r="H31" s="11" t="s">
         <v>622</v>
       </c>
-      <c r="I31" s="3" t="s">
+      <c r="I31" s="11" t="s">
         <v>387</v>
       </c>
-      <c r="J31" s="3" t="s">
+      <c r="J31" s="11" t="s">
         <v>352</v>
       </c>
-      <c r="K31" s="3" t="s">
+      <c r="K31" s="11" t="s">
         <v>688</v>
       </c>
-      <c r="L31" s="3" t="s">
+      <c r="L31" s="11" t="s">
         <v>697</v>
       </c>
     </row>
-    <row r="32" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A32" s="3" t="s">
+    <row r="32" spans="1:12" s="11" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A32" s="11" t="s">
         <v>35</v>
       </c>
-      <c r="B32" s="3" t="s">
+      <c r="B32" s="11" t="s">
         <v>474</v>
       </c>
-      <c r="C32" s="3">
+      <c r="C32" s="11">
         <f t="shared" si="0"/>
-        <v>-1E-4</v>
-      </c>
-      <c r="D32" s="3" t="s">
+        <v>-0.2</v>
+      </c>
+      <c r="D32" s="11" t="s">
         <v>589</v>
       </c>
-      <c r="E32" s="3">
-        <v>1</v>
-      </c>
-      <c r="F32" s="3" t="s">
+      <c r="E32" s="11">
+        <v>1</v>
+      </c>
+      <c r="F32" s="11" t="s">
         <v>241</v>
       </c>
-      <c r="G32" s="3" t="b">
+      <c r="G32" s="11" t="b">
         <v>0</v>
       </c>
-      <c r="H32" s="3" t="s">
+      <c r="H32" s="11" t="s">
         <v>622</v>
       </c>
-      <c r="I32" s="3" t="s">
+      <c r="I32" s="11" t="s">
         <v>387</v>
       </c>
-      <c r="J32" s="3" t="s">
+      <c r="J32" s="11" t="s">
         <v>352</v>
       </c>
-      <c r="K32" s="3" t="s">
+      <c r="K32" s="11" t="s">
         <v>688</v>
       </c>
-      <c r="L32" s="3" t="s">
+      <c r="L32" s="11" t="s">
         <v>697</v>
       </c>
     </row>
-    <row r="33" spans="1:12" s="9" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A33" s="9" t="s">
+    <row r="33" spans="1:12" s="11" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A33" s="11" t="s">
         <v>36</v>
       </c>
-      <c r="B33" s="9" t="s">
+      <c r="B33" s="11" t="s">
         <v>475</v>
       </c>
-      <c r="C33" s="9">
+      <c r="C33" s="11">
         <f t="shared" si="0"/>
-        <v>-1E-4</v>
-      </c>
-      <c r="D33" s="9" t="s">
+        <v>-0.2</v>
+      </c>
+      <c r="D33" s="11" t="s">
         <v>589</v>
       </c>
-      <c r="E33" s="9">
-        <v>1</v>
-      </c>
-      <c r="F33" s="9" t="s">
+      <c r="E33" s="11">
+        <v>1</v>
+      </c>
+      <c r="F33" s="11" t="s">
         <v>242</v>
       </c>
-      <c r="G33" s="9" t="b">
+      <c r="G33" s="11" t="b">
         <v>0</v>
       </c>
-      <c r="H33" s="9" t="s">
+      <c r="H33" s="11" t="s">
         <v>623</v>
       </c>
-      <c r="I33" s="9" t="s">
+      <c r="I33" s="11" t="s">
         <v>387</v>
       </c>
-      <c r="J33" s="9" t="s">
+      <c r="J33" s="11" t="s">
         <v>352</v>
       </c>
-      <c r="K33" s="9" t="s">
+      <c r="K33" s="11" t="s">
         <v>688</v>
       </c>
-      <c r="L33" s="9" t="s">
+      <c r="L33" s="11" t="s">
         <v>697</v>
       </c>
     </row>
@@ -18202,497 +18210,497 @@
         <v>699</v>
       </c>
     </row>
-    <row r="44" spans="1:12" s="11" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A44" s="11" t="s">
+    <row r="44" spans="1:12" s="10" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A44" s="10" t="s">
         <v>47</v>
       </c>
-      <c r="B44" s="11" t="s">
+      <c r="B44" s="10" t="s">
         <v>486</v>
       </c>
-      <c r="C44" s="11">
+      <c r="C44" s="10">
         <v>600</v>
       </c>
-      <c r="D44" s="11" t="s">
+      <c r="D44" s="10" t="s">
         <v>591</v>
       </c>
-      <c r="E44" s="11">
-        <v>1</v>
-      </c>
-      <c r="F44" s="11" t="s">
+      <c r="E44" s="10">
+        <v>1</v>
+      </c>
+      <c r="F44" s="10" t="s">
         <v>253</v>
       </c>
-      <c r="G44" s="11" t="b">
+      <c r="G44" s="10" t="b">
         <v>0</v>
       </c>
-      <c r="H44" s="11" t="s">
+      <c r="H44" s="10" t="s">
         <v>630</v>
       </c>
-      <c r="I44" s="11" t="s">
+      <c r="I44" s="10" t="s">
         <v>679</v>
       </c>
-      <c r="J44" s="11" t="s">
+      <c r="J44" s="10" t="s">
         <v>353</v>
       </c>
-      <c r="K44" s="11" t="s">
+      <c r="K44" s="10" t="s">
         <v>688</v>
       </c>
-      <c r="L44" s="11" t="s">
+      <c r="L44" s="10" t="s">
         <v>699</v>
       </c>
     </row>
-    <row r="45" spans="1:12" s="11" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A45" s="11" t="s">
+    <row r="45" spans="1:12" s="10" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A45" s="10" t="s">
         <v>48</v>
       </c>
-      <c r="B45" s="11" t="s">
+      <c r="B45" s="10" t="s">
         <v>487</v>
       </c>
-      <c r="C45" s="11">
+      <c r="C45" s="10">
         <v>170</v>
       </c>
-      <c r="D45" s="11" t="s">
+      <c r="D45" s="10" t="s">
         <v>591</v>
       </c>
-      <c r="E45" s="11">
-        <v>1</v>
-      </c>
-      <c r="F45" s="11" t="s">
+      <c r="E45" s="10">
+        <v>1</v>
+      </c>
+      <c r="F45" s="10" t="s">
         <v>254</v>
       </c>
-      <c r="G45" s="11" t="b">
+      <c r="G45" s="10" t="b">
         <v>0</v>
       </c>
-      <c r="H45" s="11" t="s">
+      <c r="H45" s="10" t="s">
         <v>631</v>
       </c>
-      <c r="I45" s="11" t="s">
+      <c r="I45" s="10" t="s">
         <v>679</v>
       </c>
-      <c r="J45" s="11" t="s">
+      <c r="J45" s="10" t="s">
         <v>353</v>
       </c>
-      <c r="K45" s="11" t="s">
+      <c r="K45" s="10" t="s">
         <v>688</v>
       </c>
-      <c r="L45" s="11" t="s">
+      <c r="L45" s="10" t="s">
         <v>699</v>
       </c>
     </row>
-    <row r="46" spans="1:12" s="11" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A46" s="11" t="s">
+    <row r="46" spans="1:12" s="10" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A46" s="10" t="s">
         <v>49</v>
       </c>
-      <c r="B46" s="11" t="s">
+      <c r="B46" s="10" t="s">
         <v>488</v>
       </c>
-      <c r="C46" s="11">
+      <c r="C46" s="10">
         <v>285</v>
       </c>
-      <c r="D46" s="11" t="s">
+      <c r="D46" s="10" t="s">
         <v>591</v>
       </c>
-      <c r="E46" s="11">
-        <v>1</v>
-      </c>
-      <c r="F46" s="11" t="s">
+      <c r="E46" s="10">
+        <v>1</v>
+      </c>
+      <c r="F46" s="10" t="s">
         <v>255</v>
       </c>
-      <c r="G46" s="11" t="b">
+      <c r="G46" s="10" t="b">
         <v>0</v>
       </c>
-      <c r="H46" s="11" t="s">
+      <c r="H46" s="10" t="s">
         <v>632</v>
       </c>
-      <c r="I46" s="11" t="s">
+      <c r="I46" s="10" t="s">
         <v>679</v>
       </c>
-      <c r="J46" s="11" t="s">
+      <c r="J46" s="10" t="s">
         <v>353</v>
       </c>
-      <c r="K46" s="11" t="s">
+      <c r="K46" s="10" t="s">
         <v>688</v>
       </c>
-      <c r="L46" s="11" t="s">
+      <c r="L46" s="10" t="s">
         <v>699</v>
       </c>
     </row>
-    <row r="47" spans="1:12" s="11" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A47" s="11" t="s">
+    <row r="47" spans="1:12" s="10" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A47" s="10" t="s">
         <v>50</v>
       </c>
-      <c r="B47" s="11" t="s">
+      <c r="B47" s="10" t="s">
         <v>489</v>
       </c>
-      <c r="C47" s="11">
+      <c r="C47" s="10">
         <v>300</v>
       </c>
-      <c r="D47" s="11" t="s">
+      <c r="D47" s="10" t="s">
         <v>591</v>
       </c>
-      <c r="E47" s="11">
-        <v>1</v>
-      </c>
-      <c r="F47" s="11" t="s">
+      <c r="E47" s="10">
+        <v>1</v>
+      </c>
+      <c r="F47" s="10" t="s">
         <v>256</v>
       </c>
-      <c r="G47" s="11" t="b">
+      <c r="G47" s="10" t="b">
         <v>0</v>
       </c>
-      <c r="H47" s="11" t="s">
+      <c r="H47" s="10" t="s">
         <v>633</v>
       </c>
-      <c r="I47" s="11" t="s">
+      <c r="I47" s="10" t="s">
         <v>679</v>
       </c>
-      <c r="J47" s="11" t="s">
+      <c r="J47" s="10" t="s">
         <v>353</v>
       </c>
-      <c r="K47" s="11" t="s">
+      <c r="K47" s="10" t="s">
         <v>688</v>
       </c>
-      <c r="L47" s="11" t="s">
+      <c r="L47" s="10" t="s">
         <v>699</v>
       </c>
     </row>
-    <row r="48" spans="1:12" s="11" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A48" s="11" t="s">
+    <row r="48" spans="1:12" s="10" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A48" s="10" t="s">
         <v>51</v>
       </c>
-      <c r="B48" s="11" t="s">
+      <c r="B48" s="10" t="s">
         <v>490</v>
       </c>
-      <c r="C48" s="11">
+      <c r="C48" s="10">
         <v>300</v>
       </c>
-      <c r="D48" s="11" t="s">
+      <c r="D48" s="10" t="s">
         <v>591</v>
       </c>
-      <c r="E48" s="11">
-        <v>1</v>
-      </c>
-      <c r="F48" s="11" t="s">
+      <c r="E48" s="10">
+        <v>1</v>
+      </c>
+      <c r="F48" s="10" t="s">
         <v>257</v>
       </c>
-      <c r="G48" s="11" t="b">
+      <c r="G48" s="10" t="b">
         <v>0</v>
       </c>
-      <c r="H48" s="11" t="s">
+      <c r="H48" s="10" t="s">
         <v>630</v>
       </c>
-      <c r="I48" s="11" t="s">
+      <c r="I48" s="10" t="s">
         <v>679</v>
       </c>
-      <c r="J48" s="11" t="s">
+      <c r="J48" s="10" t="s">
         <v>353</v>
       </c>
-      <c r="K48" s="11" t="s">
+      <c r="K48" s="10" t="s">
         <v>688</v>
       </c>
-      <c r="L48" s="11" t="s">
+      <c r="L48" s="10" t="s">
         <v>699</v>
       </c>
     </row>
-    <row r="49" spans="1:12" s="11" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A49" s="11" t="s">
+    <row r="49" spans="1:12" s="10" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A49" s="10" t="s">
         <v>52</v>
       </c>
-      <c r="B49" s="11" t="s">
+      <c r="B49" s="10" t="s">
         <v>491</v>
       </c>
-      <c r="C49" s="11">
+      <c r="C49" s="10">
         <v>500</v>
       </c>
-      <c r="D49" s="11" t="s">
+      <c r="D49" s="10" t="s">
         <v>591</v>
       </c>
-      <c r="E49" s="11">
-        <v>1</v>
-      </c>
-      <c r="F49" s="11" t="s">
+      <c r="E49" s="10">
+        <v>1</v>
+      </c>
+      <c r="F49" s="10" t="s">
         <v>258</v>
       </c>
-      <c r="G49" s="11" t="b">
+      <c r="G49" s="10" t="b">
         <v>0</v>
       </c>
-      <c r="H49" s="11" t="s">
+      <c r="H49" s="10" t="s">
         <v>634</v>
       </c>
-      <c r="I49" s="11" t="s">
+      <c r="I49" s="10" t="s">
         <v>679</v>
       </c>
-      <c r="J49" s="11" t="s">
+      <c r="J49" s="10" t="s">
         <v>353</v>
       </c>
-      <c r="K49" s="11" t="s">
+      <c r="K49" s="10" t="s">
         <v>688</v>
       </c>
-      <c r="L49" s="11" t="s">
+      <c r="L49" s="10" t="s">
         <v>699</v>
       </c>
     </row>
-    <row r="50" spans="1:12" s="11" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A50" s="11" t="s">
+    <row r="50" spans="1:12" s="10" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A50" s="10" t="s">
         <v>53</v>
       </c>
-      <c r="B50" s="11" t="s">
+      <c r="B50" s="10" t="s">
         <v>492</v>
       </c>
-      <c r="C50" s="11">
+      <c r="C50" s="10">
         <v>300</v>
       </c>
-      <c r="D50" s="11" t="s">
+      <c r="D50" s="10" t="s">
         <v>591</v>
       </c>
-      <c r="E50" s="11">
-        <v>1</v>
-      </c>
-      <c r="F50" s="11" t="s">
+      <c r="E50" s="10">
+        <v>1</v>
+      </c>
+      <c r="F50" s="10" t="s">
         <v>259</v>
       </c>
-      <c r="G50" s="11" t="b">
+      <c r="G50" s="10" t="b">
         <v>0</v>
       </c>
-      <c r="H50" s="11" t="s">
+      <c r="H50" s="10" t="s">
         <v>630</v>
       </c>
-      <c r="I50" s="11" t="s">
+      <c r="I50" s="10" t="s">
         <v>679</v>
       </c>
-      <c r="J50" s="11" t="s">
+      <c r="J50" s="10" t="s">
         <v>353</v>
       </c>
-      <c r="K50" s="11" t="s">
+      <c r="K50" s="10" t="s">
         <v>688</v>
       </c>
-      <c r="L50" s="11" t="s">
+      <c r="L50" s="10" t="s">
         <v>699</v>
       </c>
     </row>
-    <row r="51" spans="1:12" s="11" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A51" s="11" t="s">
+    <row r="51" spans="1:12" s="10" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A51" s="10" t="s">
         <v>54</v>
       </c>
-      <c r="B51" s="11" t="s">
+      <c r="B51" s="10" t="s">
         <v>493</v>
       </c>
-      <c r="C51" s="11">
+      <c r="C51" s="10">
         <v>400</v>
       </c>
-      <c r="D51" s="11" t="s">
+      <c r="D51" s="10" t="s">
         <v>591</v>
       </c>
-      <c r="E51" s="11">
-        <v>1</v>
-      </c>
-      <c r="F51" s="11" t="s">
+      <c r="E51" s="10">
+        <v>1</v>
+      </c>
+      <c r="F51" s="10" t="s">
         <v>260</v>
       </c>
-      <c r="G51" s="11" t="b">
+      <c r="G51" s="10" t="b">
         <v>0</v>
       </c>
-      <c r="H51" s="11" t="s">
+      <c r="H51" s="10" t="s">
         <v>630</v>
       </c>
-      <c r="I51" s="11" t="s">
+      <c r="I51" s="10" t="s">
         <v>679</v>
       </c>
-      <c r="J51" s="11" t="s">
+      <c r="J51" s="10" t="s">
         <v>353</v>
       </c>
-      <c r="K51" s="11" t="s">
+      <c r="K51" s="10" t="s">
         <v>688</v>
       </c>
-      <c r="L51" s="11" t="s">
+      <c r="L51" s="10" t="s">
         <v>699</v>
       </c>
     </row>
-    <row r="52" spans="1:12" s="11" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A52" s="11" t="s">
+    <row r="52" spans="1:12" s="10" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A52" s="10" t="s">
         <v>55</v>
       </c>
-      <c r="B52" s="11" t="s">
+      <c r="B52" s="10" t="s">
         <v>494</v>
       </c>
-      <c r="C52" s="11">
+      <c r="C52" s="10">
         <v>500</v>
       </c>
-      <c r="D52" s="11" t="s">
+      <c r="D52" s="10" t="s">
         <v>591</v>
       </c>
-      <c r="E52" s="11">
-        <v>1</v>
-      </c>
-      <c r="F52" s="11" t="s">
+      <c r="E52" s="10">
+        <v>1</v>
+      </c>
+      <c r="F52" s="10" t="s">
         <v>261</v>
       </c>
-      <c r="G52" s="11" t="b">
+      <c r="G52" s="10" t="b">
         <v>0</v>
       </c>
-      <c r="H52" s="11" t="s">
+      <c r="H52" s="10" t="s">
         <v>635</v>
       </c>
-      <c r="I52" s="11" t="s">
+      <c r="I52" s="10" t="s">
         <v>679</v>
       </c>
-      <c r="J52" s="11" t="s">
+      <c r="J52" s="10" t="s">
         <v>353</v>
       </c>
-      <c r="K52" s="11" t="s">
+      <c r="K52" s="10" t="s">
         <v>688</v>
       </c>
-      <c r="L52" s="11" t="s">
+      <c r="L52" s="10" t="s">
         <v>699</v>
       </c>
     </row>
-    <row r="53" spans="1:12" s="11" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A53" s="11" t="s">
+    <row r="53" spans="1:12" s="10" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A53" s="10" t="s">
         <v>56</v>
       </c>
-      <c r="B53" s="11" t="s">
+      <c r="B53" s="10" t="s">
         <v>495</v>
       </c>
-      <c r="C53" s="11">
+      <c r="C53" s="10">
         <v>300</v>
       </c>
-      <c r="D53" s="11" t="s">
+      <c r="D53" s="10" t="s">
         <v>591</v>
       </c>
-      <c r="E53" s="11">
-        <v>1</v>
-      </c>
-      <c r="F53" s="11" t="s">
+      <c r="E53" s="10">
+        <v>1</v>
+      </c>
+      <c r="F53" s="10" t="s">
         <v>262</v>
       </c>
-      <c r="G53" s="11" t="b">
+      <c r="G53" s="10" t="b">
         <v>0</v>
       </c>
-      <c r="H53" s="11" t="s">
+      <c r="H53" s="10" t="s">
         <v>636</v>
       </c>
-      <c r="I53" s="11" t="s">
+      <c r="I53" s="10" t="s">
         <v>679</v>
       </c>
-      <c r="J53" s="11" t="s">
+      <c r="J53" s="10" t="s">
         <v>353</v>
       </c>
-      <c r="K53" s="11" t="s">
+      <c r="K53" s="10" t="s">
         <v>688</v>
       </c>
-      <c r="L53" s="11" t="s">
+      <c r="L53" s="10" t="s">
         <v>699</v>
       </c>
     </row>
-    <row r="54" spans="1:12" s="11" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A54" s="11" t="s">
+    <row r="54" spans="1:12" s="10" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A54" s="10" t="s">
         <v>57</v>
       </c>
-      <c r="B54" s="11" t="s">
+      <c r="B54" s="10" t="s">
         <v>496</v>
       </c>
-      <c r="C54" s="11">
+      <c r="C54" s="10">
         <v>30</v>
       </c>
-      <c r="D54" s="11" t="s">
+      <c r="D54" s="10" t="s">
         <v>591</v>
       </c>
-      <c r="E54" s="11">
-        <v>1</v>
-      </c>
-      <c r="F54" s="11" t="s">
+      <c r="E54" s="10">
+        <v>1</v>
+      </c>
+      <c r="F54" s="10" t="s">
         <v>263</v>
       </c>
-      <c r="G54" s="11" t="b">
+      <c r="G54" s="10" t="b">
         <v>0</v>
       </c>
-      <c r="H54" s="11" t="s">
+      <c r="H54" s="10" t="s">
         <v>637</v>
       </c>
-      <c r="I54" s="11" t="s">
+      <c r="I54" s="10" t="s">
         <v>679</v>
       </c>
-      <c r="J54" s="11" t="s">
+      <c r="J54" s="10" t="s">
         <v>353</v>
       </c>
-      <c r="K54" s="11" t="s">
+      <c r="K54" s="10" t="s">
         <v>688</v>
       </c>
-      <c r="L54" s="11" t="s">
+      <c r="L54" s="10" t="s">
         <v>699</v>
       </c>
     </row>
-    <row r="55" spans="1:12" s="11" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A55" s="11" t="s">
+    <row r="55" spans="1:12" s="10" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A55" s="10" t="s">
         <v>58</v>
       </c>
-      <c r="B55" s="11" t="s">
+      <c r="B55" s="10" t="s">
         <v>497</v>
       </c>
-      <c r="C55" s="11">
+      <c r="C55" s="10">
         <v>300</v>
       </c>
-      <c r="D55" s="11" t="s">
+      <c r="D55" s="10" t="s">
         <v>591</v>
       </c>
-      <c r="E55" s="11">
-        <v>1</v>
-      </c>
-      <c r="F55" s="11" t="s">
+      <c r="E55" s="10">
+        <v>1</v>
+      </c>
+      <c r="F55" s="10" t="s">
         <v>264</v>
       </c>
-      <c r="G55" s="11" t="b">
+      <c r="G55" s="10" t="b">
         <v>0</v>
       </c>
-      <c r="H55" s="11" t="s">
+      <c r="H55" s="10" t="s">
         <v>638</v>
       </c>
-      <c r="I55" s="11" t="s">
+      <c r="I55" s="10" t="s">
         <v>679</v>
       </c>
-      <c r="J55" s="11" t="s">
+      <c r="J55" s="10" t="s">
         <v>353</v>
       </c>
-      <c r="K55" s="11" t="s">
+      <c r="K55" s="10" t="s">
         <v>688</v>
       </c>
-      <c r="L55" s="11" t="s">
+      <c r="L55" s="10" t="s">
         <v>699</v>
       </c>
     </row>
-    <row r="56" spans="1:12" s="11" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A56" s="11" t="s">
+    <row r="56" spans="1:12" s="10" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A56" s="10" t="s">
         <v>59</v>
       </c>
-      <c r="B56" s="11" t="s">
+      <c r="B56" s="10" t="s">
         <v>498</v>
       </c>
-      <c r="C56" s="11">
+      <c r="C56" s="10">
         <v>300</v>
       </c>
-      <c r="D56" s="11" t="s">
+      <c r="D56" s="10" t="s">
         <v>591</v>
       </c>
-      <c r="E56" s="11">
-        <v>1</v>
-      </c>
-      <c r="F56" s="11" t="s">
+      <c r="E56" s="10">
+        <v>1</v>
+      </c>
+      <c r="F56" s="10" t="s">
         <v>265</v>
       </c>
-      <c r="G56" s="11" t="b">
+      <c r="G56" s="10" t="b">
         <v>0</v>
       </c>
-      <c r="H56" s="11" t="s">
+      <c r="H56" s="10" t="s">
         <v>639</v>
       </c>
-      <c r="I56" s="11" t="s">
+      <c r="I56" s="10" t="s">
         <v>679</v>
       </c>
-      <c r="J56" s="11" t="s">
+      <c r="J56" s="10" t="s">
         <v>353</v>
       </c>
-      <c r="K56" s="11" t="s">
+      <c r="K56" s="10" t="s">
         <v>688</v>
       </c>
-      <c r="L56" s="11" t="s">
+      <c r="L56" s="10" t="s">
         <v>699</v>
       </c>
     </row>
@@ -19496,41 +19504,41 @@
         <v>706</v>
       </c>
     </row>
-    <row r="78" spans="1:12" s="5" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A78" s="5" t="s">
+    <row r="78" spans="1:12" s="11" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A78" s="11" t="s">
         <v>81</v>
       </c>
-      <c r="B78" s="5" t="s">
+      <c r="B78" s="11" t="s">
         <v>517</v>
       </c>
-      <c r="C78" s="5">
-        <v>-130</v>
-      </c>
-      <c r="D78" s="5" t="s">
+      <c r="C78" s="11">
+        <v>-1500</v>
+      </c>
+      <c r="D78" s="11" t="s">
         <v>588</v>
       </c>
-      <c r="E78" s="5">
-        <v>1</v>
-      </c>
-      <c r="F78" s="5" t="s">
+      <c r="E78" s="11">
+        <v>1</v>
+      </c>
+      <c r="F78" s="11" t="s">
         <v>266</v>
       </c>
-      <c r="G78" s="5" t="b">
-        <v>1</v>
-      </c>
-      <c r="H78" s="5" t="s">
+      <c r="G78" s="11" t="b">
+        <v>1</v>
+      </c>
+      <c r="H78" s="11" t="s">
         <v>653</v>
       </c>
-      <c r="I78" s="5" t="s">
+      <c r="I78" s="11" t="s">
         <v>395</v>
       </c>
-      <c r="J78" s="5" t="s">
+      <c r="J78" s="11" t="s">
         <v>356</v>
       </c>
-      <c r="K78" s="5" t="s">
+      <c r="K78" s="11" t="s">
         <v>688</v>
       </c>
-      <c r="L78" s="5" t="s">
+      <c r="L78" s="11" t="s">
         <v>707</v>
       </c>
     </row>
@@ -19954,79 +19962,79 @@
         <v>709</v>
       </c>
     </row>
-    <row r="90" spans="1:12" s="6" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A90" s="6" t="s">
+    <row r="90" spans="1:12" s="5" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A90" s="5" t="s">
         <v>93</v>
       </c>
-      <c r="B90" s="6" t="s">
+      <c r="B90" s="5" t="s">
         <v>464</v>
       </c>
-      <c r="C90" s="6">
+      <c r="C90" s="5">
         <v>-20</v>
       </c>
-      <c r="D90" s="6" t="s">
+      <c r="D90" s="5" t="s">
         <v>588</v>
       </c>
-      <c r="E90" s="6">
-        <v>1</v>
-      </c>
-      <c r="F90" s="6" t="s">
+      <c r="E90" s="5">
+        <v>1</v>
+      </c>
+      <c r="F90" s="5" t="s">
         <v>287</v>
       </c>
-      <c r="G90" s="6" t="b">
-        <v>1</v>
-      </c>
-      <c r="H90" s="6" t="s">
+      <c r="G90" s="5" t="b">
+        <v>1</v>
+      </c>
+      <c r="H90" s="5" t="s">
         <v>662</v>
       </c>
-      <c r="I90" s="6" t="s">
+      <c r="I90" s="5" t="s">
         <v>398</v>
       </c>
-      <c r="J90" s="6" t="s">
+      <c r="J90" s="5" t="s">
         <v>350</v>
       </c>
-      <c r="K90" s="6" t="s">
+      <c r="K90" s="5" t="s">
         <v>688</v>
       </c>
-      <c r="L90" s="6" t="s">
+      <c r="L90" s="5" t="s">
         <v>710</v>
       </c>
     </row>
-    <row r="91" spans="1:12" s="6" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A91" s="6" t="s">
+    <row r="91" spans="1:12" s="5" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A91" s="5" t="s">
         <v>94</v>
       </c>
-      <c r="B91" s="6" t="s">
+      <c r="B91" s="5" t="s">
         <v>465</v>
       </c>
-      <c r="C91" s="6">
+      <c r="C91" s="5">
         <v>-20</v>
       </c>
-      <c r="D91" s="6" t="s">
+      <c r="D91" s="5" t="s">
         <v>588</v>
       </c>
-      <c r="E91" s="6">
-        <v>1</v>
-      </c>
-      <c r="F91" s="6" t="s">
+      <c r="E91" s="5">
+        <v>1</v>
+      </c>
+      <c r="F91" s="5" t="s">
         <v>288</v>
       </c>
-      <c r="G91" s="6" t="b">
-        <v>1</v>
-      </c>
-      <c r="H91" s="6" t="s">
+      <c r="G91" s="5" t="b">
+        <v>1</v>
+      </c>
+      <c r="H91" s="5" t="s">
         <v>662</v>
       </c>
-      <c r="I91" s="6" t="s">
+      <c r="I91" s="5" t="s">
         <v>398</v>
       </c>
-      <c r="J91" s="6" t="s">
+      <c r="J91" s="5" t="s">
         <v>350</v>
       </c>
-      <c r="K91" s="6" t="s">
+      <c r="K91" s="5" t="s">
         <v>688</v>
       </c>
-      <c r="L91" s="6" t="s">
+      <c r="L91" s="5" t="s">
         <v>710</v>
       </c>
     </row>
@@ -20069,42 +20077,42 @@
         <v>710</v>
       </c>
     </row>
-    <row r="93" spans="1:12" s="6" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A93" s="6" t="s">
+    <row r="93" spans="1:12" s="5" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A93" s="5" t="s">
         <v>96</v>
       </c>
-      <c r="B93" s="6" t="s">
+      <c r="B93" s="5" t="s">
         <v>467</v>
       </c>
-      <c r="C93" s="6">
+      <c r="C93" s="5">
         <f>-20.0067</f>
         <v>-20.006699999999999</v>
       </c>
-      <c r="D93" s="6" t="s">
+      <c r="D93" s="5" t="s">
         <v>588</v>
       </c>
-      <c r="E93" s="6">
-        <v>1</v>
-      </c>
-      <c r="F93" s="6" t="s">
+      <c r="E93" s="5">
+        <v>1</v>
+      </c>
+      <c r="F93" s="5" t="s">
         <v>290</v>
       </c>
-      <c r="G93" s="6" t="b">
-        <v>1</v>
-      </c>
-      <c r="H93" s="6" t="s">
+      <c r="G93" s="5" t="b">
+        <v>1</v>
+      </c>
+      <c r="H93" s="5" t="s">
         <v>662</v>
       </c>
-      <c r="I93" s="6" t="s">
+      <c r="I93" s="5" t="s">
         <v>398</v>
       </c>
-      <c r="J93" s="6" t="s">
+      <c r="J93" s="5" t="s">
         <v>350</v>
       </c>
-      <c r="K93" s="6" t="s">
+      <c r="K93" s="5" t="s">
         <v>688</v>
       </c>
-      <c r="L93" s="6" t="s">
+      <c r="L93" s="5" t="s">
         <v>710</v>
       </c>
     </row>
@@ -20186,41 +20194,41 @@
         <v>710</v>
       </c>
     </row>
-    <row r="96" spans="1:12" s="6" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A96" s="6" t="s">
+    <row r="96" spans="1:12" s="5" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A96" s="5" t="s">
         <v>99</v>
       </c>
-      <c r="B96" s="6" t="s">
+      <c r="B96" s="5" t="s">
         <v>524</v>
       </c>
-      <c r="C96" s="6">
+      <c r="C96" s="5">
         <v>-10000</v>
       </c>
-      <c r="D96" s="6" t="s">
+      <c r="D96" s="5" t="s">
         <v>597</v>
       </c>
-      <c r="E96" s="6">
-        <v>1</v>
-      </c>
-      <c r="F96" s="6" t="s">
+      <c r="E96" s="5">
+        <v>1</v>
+      </c>
+      <c r="F96" s="5" t="s">
         <v>293</v>
       </c>
-      <c r="G96" s="6" t="b">
+      <c r="G96" s="5" t="b">
         <v>0</v>
       </c>
-      <c r="H96" s="6" t="s">
+      <c r="H96" s="5" t="s">
         <v>663</v>
       </c>
-      <c r="I96" s="6" t="s">
+      <c r="I96" s="5" t="s">
         <v>399</v>
       </c>
-      <c r="J96" s="6" t="s">
+      <c r="J96" s="5" t="s">
         <v>351</v>
       </c>
-      <c r="K96" s="6" t="s">
+      <c r="K96" s="5" t="s">
         <v>688</v>
       </c>
-      <c r="L96" s="6" t="s">
+      <c r="L96" s="5" t="s">
         <v>711</v>
       </c>
     </row>
@@ -22678,7 +22686,7 @@
     <col min="6" max="6" width="26.83203125" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="37.6640625" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="84.83203125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="10.6640625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="11.1640625" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="20.33203125" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="9" bestFit="1" customWidth="1"/>
     <col min="13" max="14" width="9" bestFit="1" customWidth="1"/>
@@ -23813,50 +23821,50 @@
         <v>824</v>
       </c>
     </row>
-    <row r="25" spans="1:15" s="9" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A25" s="9" t="s">
+    <row r="25" spans="1:15" s="8" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A25" s="8" t="s">
         <v>2046</v>
       </c>
-      <c r="B25" s="9" t="s">
+      <c r="B25" s="8" t="s">
         <v>737</v>
       </c>
-      <c r="C25" s="9" t="b">
-        <v>1</v>
-      </c>
-      <c r="D25" s="9">
+      <c r="C25" s="8" t="b">
+        <v>1</v>
+      </c>
+      <c r="D25" s="8">
         <v>99</v>
       </c>
-      <c r="E25" s="9" t="s">
+      <c r="E25" s="8" t="s">
         <v>350</v>
       </c>
-      <c r="F25" s="9" t="s">
+      <c r="F25" s="8" t="s">
         <v>350</v>
       </c>
-      <c r="G25" s="9" t="s">
+      <c r="G25" s="8" t="s">
         <v>767</v>
       </c>
-      <c r="H25" s="9" t="s">
+      <c r="H25" s="8" t="s">
         <v>2047</v>
       </c>
-      <c r="I25" s="9">
+      <c r="I25" s="8">
         <v>5</v>
       </c>
-      <c r="J25" s="9" t="s">
+      <c r="J25" s="8" t="s">
         <v>797</v>
       </c>
-      <c r="K25" s="9">
-        <v>1</v>
-      </c>
-      <c r="L25" s="9" t="s">
+      <c r="K25" s="8">
+        <v>1</v>
+      </c>
+      <c r="L25" s="8" t="s">
         <v>350</v>
       </c>
-      <c r="M25" s="9">
+      <c r="M25" s="8">
         <v>99</v>
       </c>
-      <c r="N25" s="9" t="b">
+      <c r="N25" s="8" t="b">
         <v>0</v>
       </c>
-      <c r="O25" s="9" t="s">
+      <c r="O25" s="8" t="s">
         <v>825</v>
       </c>
     </row>
@@ -23907,97 +23915,97 @@
         <v>826</v>
       </c>
     </row>
-    <row r="27" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A27" t="s">
+    <row r="27" spans="1:15" s="11" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A27" s="11" t="s">
         <v>188</v>
       </c>
-      <c r="B27" t="s">
+      <c r="B27" s="11" t="s">
         <v>739</v>
       </c>
-      <c r="C27" t="b">
-        <v>1</v>
-      </c>
-      <c r="D27">
+      <c r="C27" s="11" t="b">
+        <v>1</v>
+      </c>
+      <c r="D27" s="11">
         <v>99</v>
       </c>
-      <c r="E27" t="s">
+      <c r="E27" s="11" t="s">
         <v>350</v>
       </c>
-      <c r="F27" t="s">
+      <c r="F27" s="11" t="s">
         <v>350</v>
       </c>
-      <c r="G27" t="s">
+      <c r="G27" s="11" t="s">
         <v>765</v>
       </c>
-      <c r="H27" t="s">
+      <c r="H27" s="11" t="s">
         <v>785</v>
       </c>
-      <c r="I27">
-        <v>13000000</v>
-      </c>
-      <c r="J27" t="s">
+      <c r="I27" s="11">
+        <v>30000000</v>
+      </c>
+      <c r="J27" s="11" t="s">
         <v>798</v>
       </c>
-      <c r="K27">
-        <v>1</v>
-      </c>
-      <c r="L27" t="s">
+      <c r="K27" s="11">
+        <v>1</v>
+      </c>
+      <c r="L27" s="11" t="s">
         <v>806</v>
       </c>
-      <c r="M27">
-        <v>1</v>
-      </c>
-      <c r="N27" t="b">
-        <v>1</v>
-      </c>
-      <c r="O27" t="s">
+      <c r="M27" s="11">
+        <v>1</v>
+      </c>
+      <c r="N27" s="11" t="b">
+        <v>1</v>
+      </c>
+      <c r="O27" s="11" t="s">
         <v>827</v>
       </c>
     </row>
-    <row r="28" spans="1:15" s="7" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A28" s="7" t="s">
+    <row r="28" spans="1:15" s="6" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A28" s="6" t="s">
         <v>189</v>
       </c>
-      <c r="B28" s="7" t="s">
+      <c r="B28" s="6" t="s">
         <v>740</v>
       </c>
-      <c r="C28" s="7" t="b">
-        <v>1</v>
-      </c>
-      <c r="D28" s="7">
+      <c r="C28" s="6" t="b">
+        <v>1</v>
+      </c>
+      <c r="D28" s="6">
         <v>99</v>
       </c>
-      <c r="E28" s="7" t="s">
+      <c r="E28" s="6" t="s">
         <v>350</v>
       </c>
-      <c r="F28" s="7" t="s">
+      <c r="F28" s="6" t="s">
         <v>350</v>
       </c>
-      <c r="G28" s="7" t="s">
+      <c r="G28" s="6" t="s">
         <v>765</v>
       </c>
-      <c r="H28" s="7" t="s">
+      <c r="H28" s="6" t="s">
         <v>786</v>
       </c>
-      <c r="I28" s="7">
+      <c r="I28" s="6">
         <v>15000000</v>
       </c>
-      <c r="J28" s="7" t="s">
+      <c r="J28" s="6" t="s">
         <v>798</v>
       </c>
-      <c r="K28" s="7">
-        <v>1</v>
-      </c>
-      <c r="L28" s="7" t="s">
+      <c r="K28" s="6">
+        <v>1</v>
+      </c>
+      <c r="L28" s="6" t="s">
         <v>2048</v>
       </c>
-      <c r="M28" s="7">
-        <v>1</v>
-      </c>
-      <c r="N28" s="7" t="b">
+      <c r="M28" s="6">
+        <v>1</v>
+      </c>
+      <c r="N28" s="6" t="b">
         <v>0</v>
       </c>
-      <c r="O28" s="7" t="s">
+      <c r="O28" s="6" t="s">
         <v>826</v>
       </c>
     </row>
@@ -24189,50 +24197,50 @@
         <v>828</v>
       </c>
     </row>
-    <row r="33" spans="1:15" s="6" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A33" s="6" t="s">
+    <row r="33" spans="1:15" s="13" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A33" s="13" t="s">
         <v>194</v>
       </c>
-      <c r="B33" s="6" t="s">
+      <c r="B33" s="13" t="s">
         <v>745</v>
       </c>
-      <c r="C33" s="6" t="b">
-        <v>1</v>
-      </c>
-      <c r="D33" s="6">
+      <c r="C33" s="13" t="b">
+        <v>1</v>
+      </c>
+      <c r="D33" s="13">
         <v>99</v>
       </c>
-      <c r="E33" s="6" t="s">
+      <c r="E33" s="13" t="s">
         <v>350</v>
       </c>
-      <c r="F33" s="6" t="s">
+      <c r="F33" s="13" t="s">
         <v>350</v>
       </c>
-      <c r="G33" s="6" t="s">
+      <c r="G33" s="13" t="s">
         <v>770</v>
       </c>
-      <c r="H33" s="6" t="s">
+      <c r="H33" s="13" t="s">
         <v>790</v>
       </c>
-      <c r="I33" s="6">
-        <v>-70</v>
-      </c>
-      <c r="J33" s="6" t="s">
+      <c r="I33" s="13">
+        <v>-300</v>
+      </c>
+      <c r="J33" s="13" t="s">
         <v>800</v>
       </c>
-      <c r="K33" s="6">
-        <v>1</v>
-      </c>
-      <c r="L33" s="6" t="s">
+      <c r="K33" s="13">
+        <v>1</v>
+      </c>
+      <c r="L33" s="13" t="s">
         <v>350</v>
       </c>
-      <c r="M33" s="6">
+      <c r="M33" s="13">
         <v>99</v>
       </c>
-      <c r="N33" s="6" t="b">
+      <c r="N33" s="13" t="b">
         <v>0</v>
       </c>
-      <c r="O33" s="6" t="s">
+      <c r="O33" s="13" t="s">
         <v>829</v>
       </c>
     </row>
@@ -24331,144 +24339,144 @@
         <v>831</v>
       </c>
     </row>
-    <row r="36" spans="1:15" s="6" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A36" s="6" t="s">
+    <row r="36" spans="1:15" s="11" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A36" s="11" t="s">
         <v>197</v>
       </c>
-      <c r="B36" s="6" t="s">
+      <c r="B36" s="11" t="s">
         <v>747</v>
       </c>
-      <c r="C36" s="6" t="b">
-        <v>1</v>
-      </c>
-      <c r="D36" s="6">
+      <c r="C36" s="11" t="b">
+        <v>1</v>
+      </c>
+      <c r="D36" s="11">
         <v>99</v>
       </c>
-      <c r="E36" s="6" t="s">
+      <c r="E36" s="11" t="s">
         <v>350</v>
       </c>
-      <c r="F36" s="6" t="s">
+      <c r="F36" s="11" t="s">
         <v>350</v>
       </c>
-      <c r="G36" s="6" t="s">
+      <c r="G36" s="11" t="s">
         <v>771</v>
       </c>
-      <c r="H36" s="6" t="s">
+      <c r="H36" s="11" t="s">
         <v>477</v>
       </c>
-      <c r="I36" s="6">
-        <v>-20</v>
-      </c>
-      <c r="J36" s="6" t="s">
+      <c r="I36" s="11">
+        <v>-27</v>
+      </c>
+      <c r="J36" s="11" t="s">
         <v>590</v>
       </c>
-      <c r="K36" s="6">
-        <v>1</v>
-      </c>
-      <c r="L36" s="6" t="s">
+      <c r="K36" s="11">
+        <v>1</v>
+      </c>
+      <c r="L36" s="11" t="s">
         <v>350</v>
       </c>
-      <c r="M36" s="6">
+      <c r="M36" s="11">
         <v>99</v>
       </c>
-      <c r="N36" s="6" t="b">
+      <c r="N36" s="11" t="b">
         <v>0</v>
       </c>
-      <c r="O36" s="6" t="s">
+      <c r="O36" s="11" t="s">
         <v>832</v>
       </c>
     </row>
-    <row r="37" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A37" t="s">
+    <row r="37" spans="1:15" s="11" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A37" s="11" t="s">
         <v>198</v>
       </c>
-      <c r="B37" t="s">
+      <c r="B37" s="11" t="s">
         <v>748</v>
       </c>
-      <c r="C37" t="b">
-        <v>1</v>
-      </c>
-      <c r="D37">
+      <c r="C37" s="11" t="b">
+        <v>1</v>
+      </c>
+      <c r="D37" s="11">
         <v>99</v>
       </c>
-      <c r="E37" t="s">
+      <c r="E37" s="11" t="s">
         <v>350</v>
       </c>
-      <c r="F37" t="s">
+      <c r="F37" s="11" t="s">
         <v>350</v>
       </c>
-      <c r="G37" t="s">
+      <c r="G37" s="11" t="s">
         <v>772</v>
       </c>
-      <c r="H37" t="s">
+      <c r="H37" s="11" t="s">
         <v>792</v>
       </c>
-      <c r="I37">
-        <v>-31</v>
-      </c>
-      <c r="J37" t="s">
+      <c r="I37" s="11">
+        <v>-120</v>
+      </c>
+      <c r="J37" s="11" t="s">
         <v>801</v>
       </c>
-      <c r="K37">
-        <v>1</v>
-      </c>
-      <c r="L37" t="s">
+      <c r="K37" s="11">
+        <v>1</v>
+      </c>
+      <c r="L37" s="11" t="s">
         <v>350</v>
       </c>
-      <c r="M37">
+      <c r="M37" s="11">
         <v>99</v>
       </c>
-      <c r="N37" t="b">
+      <c r="N37" s="11" t="b">
         <v>0</v>
       </c>
-      <c r="O37" t="s">
+      <c r="O37" s="11" t="s">
         <v>833</v>
       </c>
     </row>
-    <row r="38" spans="1:15" s="6" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A38" s="6" t="s">
+    <row r="38" spans="1:15" s="5" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A38" s="5" t="s">
         <v>199</v>
       </c>
-      <c r="B38" s="6" t="s">
+      <c r="B38" s="5" t="s">
         <v>749</v>
       </c>
-      <c r="C38" s="6" t="b">
-        <v>1</v>
-      </c>
-      <c r="D38" s="6">
+      <c r="C38" s="5" t="b">
+        <v>1</v>
+      </c>
+      <c r="D38" s="5">
         <v>99</v>
       </c>
-      <c r="E38" s="6" t="s">
+      <c r="E38" s="5" t="s">
         <v>760</v>
       </c>
-      <c r="F38" s="6" t="s">
+      <c r="F38" s="5" t="s">
         <v>762</v>
       </c>
-      <c r="G38" s="6" t="s">
+      <c r="G38" s="5" t="s">
         <v>763</v>
       </c>
-      <c r="H38" s="6" t="s">
+      <c r="H38" s="5" t="s">
         <v>793</v>
       </c>
-      <c r="I38" s="6">
+      <c r="I38" s="5">
         <v>-19</v>
       </c>
-      <c r="J38" s="6" t="s">
+      <c r="J38" s="5" t="s">
         <v>591</v>
       </c>
-      <c r="K38" s="6">
-        <v>1</v>
-      </c>
-      <c r="L38" s="6" t="s">
+      <c r="K38" s="5">
+        <v>1</v>
+      </c>
+      <c r="L38" s="5" t="s">
         <v>350</v>
       </c>
-      <c r="M38" s="6">
+      <c r="M38" s="5">
         <v>99</v>
       </c>
-      <c r="N38" s="6" t="b">
+      <c r="N38" s="5" t="b">
         <v>0</v>
       </c>
-      <c r="O38" s="6" t="s">
+      <c r="O38" s="5" t="s">
         <v>834</v>
       </c>
     </row>
@@ -24801,97 +24809,97 @@
         <v>838</v>
       </c>
     </row>
-    <row r="46" spans="1:15" s="6" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A46" s="6" t="s">
+    <row r="46" spans="1:15" s="11" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A46" s="11" t="s">
         <v>207</v>
       </c>
-      <c r="B46" s="6" t="s">
+      <c r="B46" s="11" t="s">
         <v>1887</v>
       </c>
-      <c r="C46" s="6" t="b">
-        <v>1</v>
-      </c>
-      <c r="D46" s="6">
+      <c r="C46" s="11" t="b">
+        <v>1</v>
+      </c>
+      <c r="D46" s="11">
         <v>99</v>
       </c>
-      <c r="E46" s="6" t="s">
+      <c r="E46" s="11" t="s">
         <v>760</v>
       </c>
-      <c r="F46" s="6" t="s">
+      <c r="F46" s="11" t="s">
         <v>762</v>
       </c>
-      <c r="G46" s="6" t="s">
+      <c r="G46" s="11" t="s">
         <v>763</v>
       </c>
-      <c r="H46" s="6" t="s">
+      <c r="H46" s="11" t="s">
         <v>459</v>
       </c>
-      <c r="I46" s="6">
-        <v>-81</v>
-      </c>
-      <c r="J46" s="6" t="s">
+      <c r="I46" s="11">
+        <v>-293</v>
+      </c>
+      <c r="J46" s="11" t="s">
         <v>586</v>
       </c>
-      <c r="K46" s="6">
-        <v>1</v>
-      </c>
-      <c r="L46" s="6" t="s">
+      <c r="K46" s="11">
+        <v>1</v>
+      </c>
+      <c r="L46" s="11" t="s">
         <v>350</v>
       </c>
-      <c r="M46" s="6">
+      <c r="M46" s="11">
         <v>99</v>
       </c>
-      <c r="N46" s="6" t="b">
+      <c r="N46" s="11" t="b">
         <v>0</v>
       </c>
-      <c r="O46" s="6" t="s">
+      <c r="O46" s="11" t="s">
         <v>838</v>
       </c>
     </row>
-    <row r="47" spans="1:15" s="9" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A47" s="9" t="s">
+    <row r="47" spans="1:15" s="8" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A47" s="8" t="s">
         <v>208</v>
       </c>
-      <c r="B47" s="9" t="s">
+      <c r="B47" s="8" t="s">
         <v>756</v>
       </c>
-      <c r="C47" s="9" t="b">
-        <v>1</v>
-      </c>
-      <c r="D47" s="9">
+      <c r="C47" s="8" t="b">
+        <v>1</v>
+      </c>
+      <c r="D47" s="8">
         <v>99</v>
       </c>
-      <c r="E47" s="9" t="s">
+      <c r="E47" s="8" t="s">
         <v>350</v>
       </c>
-      <c r="F47" s="9" t="s">
+      <c r="F47" s="8" t="s">
         <v>350</v>
       </c>
-      <c r="G47" s="9" t="s">
+      <c r="G47" s="8" t="s">
         <v>775</v>
       </c>
-      <c r="H47" s="9" t="s">
+      <c r="H47" s="8" t="s">
         <v>505</v>
       </c>
-      <c r="I47" s="9">
+      <c r="I47" s="8">
         <v>0</v>
       </c>
-      <c r="J47" s="9" t="s">
+      <c r="J47" s="8" t="s">
         <v>593</v>
       </c>
-      <c r="K47" s="9">
+      <c r="K47" s="8">
         <v>0</v>
       </c>
-      <c r="L47" s="9" t="s">
+      <c r="L47" s="8" t="s">
         <v>350</v>
       </c>
-      <c r="M47" s="9">
+      <c r="M47" s="8">
         <v>99</v>
       </c>
-      <c r="N47" s="9" t="b">
+      <c r="N47" s="8" t="b">
         <v>0</v>
       </c>
-      <c r="O47" s="9" t="s">
+      <c r="O47" s="8" t="s">
         <v>839</v>
       </c>
     </row>
@@ -24989,238 +24997,238 @@
         <v>841</v>
       </c>
     </row>
-    <row r="50" spans="1:15" s="9" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A50" s="9" t="s">
+    <row r="50" spans="1:15" s="11" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A50" s="11" t="s">
         <v>2038</v>
       </c>
-      <c r="B50" s="9" t="s">
+      <c r="B50" s="11" t="s">
         <v>758</v>
       </c>
-      <c r="C50" s="9" t="b">
-        <v>1</v>
-      </c>
-      <c r="D50" s="9">
+      <c r="C50" s="11" t="b">
+        <v>1</v>
+      </c>
+      <c r="D50" s="11">
         <v>99</v>
       </c>
-      <c r="E50" s="9" t="s">
+      <c r="E50" s="11" t="s">
         <v>350</v>
       </c>
-      <c r="F50" s="9" t="s">
+      <c r="F50" s="11" t="s">
         <v>350</v>
       </c>
-      <c r="G50" s="9" t="s">
+      <c r="G50" s="11" t="s">
         <v>776</v>
       </c>
-      <c r="H50" s="9" t="s">
+      <c r="H50" s="11" t="s">
         <v>2041</v>
       </c>
-      <c r="I50" s="9">
-        <v>-10</v>
-      </c>
-      <c r="J50" s="9" t="s">
+      <c r="I50" s="11">
+        <v>-20</v>
+      </c>
+      <c r="J50" s="11" t="s">
         <v>804</v>
       </c>
-      <c r="K50" s="9">
-        <v>1</v>
-      </c>
-      <c r="L50" s="9" t="s">
+      <c r="K50" s="11">
+        <v>1</v>
+      </c>
+      <c r="L50" s="11" t="s">
         <v>350</v>
       </c>
-      <c r="M50" s="9">
+      <c r="M50" s="11">
         <v>99</v>
       </c>
-      <c r="N50" s="9" t="b">
+      <c r="N50" s="11" t="b">
         <v>0</v>
       </c>
-      <c r="O50" s="9" t="s">
+      <c r="O50" s="11" t="s">
         <v>842</v>
       </c>
     </row>
-    <row r="51" spans="1:15" s="9" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A51" s="9" t="s">
+    <row r="51" spans="1:15" s="11" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A51" s="11" t="s">
         <v>2039</v>
       </c>
-      <c r="B51" s="9" t="s">
+      <c r="B51" s="11" t="s">
         <v>1891</v>
       </c>
-      <c r="C51" s="9" t="b">
-        <v>1</v>
-      </c>
-      <c r="D51" s="9">
+      <c r="C51" s="11" t="b">
+        <v>1</v>
+      </c>
+      <c r="D51" s="11">
         <v>99</v>
       </c>
-      <c r="E51" s="9" t="s">
+      <c r="E51" s="11" t="s">
         <v>350</v>
       </c>
-      <c r="F51" s="9" t="s">
+      <c r="F51" s="11" t="s">
         <v>350</v>
       </c>
-      <c r="G51" s="9" t="s">
+      <c r="G51" s="11" t="s">
         <v>776</v>
       </c>
-      <c r="H51" s="9" t="s">
+      <c r="H51" s="11" t="s">
         <v>480</v>
       </c>
-      <c r="I51" s="9">
-        <v>-0.2</v>
-      </c>
-      <c r="J51" s="9" t="s">
+      <c r="I51" s="11">
+        <v>-1</v>
+      </c>
+      <c r="J51" s="11" t="s">
         <v>804</v>
       </c>
-      <c r="K51" s="9">
-        <v>1</v>
-      </c>
-      <c r="L51" s="9" t="s">
+      <c r="K51" s="11">
+        <v>1</v>
+      </c>
+      <c r="L51" s="11" t="s">
         <v>350</v>
       </c>
-      <c r="M51" s="9">
+      <c r="M51" s="11">
         <v>99</v>
       </c>
-      <c r="N51" s="9" t="b">
+      <c r="N51" s="11" t="b">
         <v>0</v>
       </c>
-      <c r="O51" s="9" t="s">
+      <c r="O51" s="11" t="s">
         <v>842</v>
       </c>
     </row>
-    <row r="52" spans="1:15" s="9" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A52" s="9" t="s">
+    <row r="52" spans="1:15" s="11" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A52" s="11" t="s">
         <v>2040</v>
       </c>
-      <c r="B52" s="9" t="s">
+      <c r="B52" s="11" t="s">
         <v>1890</v>
       </c>
-      <c r="C52" s="9" t="b">
-        <v>1</v>
-      </c>
-      <c r="D52" s="9">
+      <c r="C52" s="11" t="b">
+        <v>1</v>
+      </c>
+      <c r="D52" s="11">
         <v>99</v>
       </c>
-      <c r="E52" s="9" t="s">
+      <c r="E52" s="11" t="s">
         <v>350</v>
       </c>
-      <c r="F52" s="9" t="s">
+      <c r="F52" s="11" t="s">
         <v>350</v>
       </c>
-      <c r="G52" s="9" t="s">
+      <c r="G52" s="11" t="s">
         <v>776</v>
       </c>
-      <c r="H52" s="9" t="s">
+      <c r="H52" s="11" t="s">
         <v>2042</v>
       </c>
-      <c r="I52" s="9">
-        <v>-0.3</v>
-      </c>
-      <c r="J52" s="9" t="s">
+      <c r="I52" s="11">
+        <v>-8</v>
+      </c>
+      <c r="J52" s="11" t="s">
         <v>804</v>
       </c>
-      <c r="K52" s="9">
-        <v>1</v>
-      </c>
-      <c r="L52" s="9" t="s">
+      <c r="K52" s="11">
+        <v>1</v>
+      </c>
+      <c r="L52" s="11" t="s">
         <v>350</v>
       </c>
-      <c r="M52" s="9">
+      <c r="M52" s="11">
         <v>99</v>
       </c>
-      <c r="N52" s="9" t="b">
+      <c r="N52" s="11" t="b">
         <v>0</v>
       </c>
-      <c r="O52" s="9" t="s">
+      <c r="O52" s="11" t="s">
         <v>842</v>
       </c>
     </row>
-    <row r="53" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A53" s="6" t="s">
+    <row r="53" spans="1:15" s="11" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A53" s="11" t="s">
         <v>2049</v>
       </c>
-      <c r="B53" s="6" t="s">
+      <c r="B53" s="11" t="s">
         <v>1889</v>
       </c>
-      <c r="C53" s="6" t="b">
-        <v>1</v>
-      </c>
-      <c r="D53" s="6">
+      <c r="C53" s="11" t="b">
+        <v>1</v>
+      </c>
+      <c r="D53" s="11">
         <v>99</v>
       </c>
-      <c r="E53" s="6" t="s">
+      <c r="E53" s="11" t="s">
         <v>350</v>
       </c>
-      <c r="F53" s="6" t="s">
+      <c r="F53" s="11" t="s">
         <v>350</v>
       </c>
-      <c r="G53" s="6" t="s">
+      <c r="G53" s="11" t="s">
         <v>763</v>
       </c>
-      <c r="H53" s="6" t="s">
+      <c r="H53" s="11" t="s">
         <v>2058</v>
       </c>
-      <c r="I53" s="6">
-        <v>20000000</v>
-      </c>
-      <c r="J53" s="6" t="s">
+      <c r="I53" s="11">
+        <v>200000000</v>
+      </c>
+      <c r="J53" s="11" t="s">
         <v>2051</v>
       </c>
-      <c r="K53" s="6">
-        <v>1</v>
-      </c>
-      <c r="L53" s="6" t="s">
+      <c r="K53" s="11">
+        <v>1</v>
+      </c>
+      <c r="L53" s="11" t="s">
         <v>350</v>
       </c>
-      <c r="M53" s="6">
+      <c r="M53" s="11">
         <v>99</v>
       </c>
-      <c r="N53" s="6" t="b">
+      <c r="N53" s="11" t="b">
         <v>0</v>
       </c>
-      <c r="O53" s="6" t="s">
+      <c r="O53" s="11" t="s">
         <v>2052</v>
       </c>
     </row>
     <row r="54" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A54" s="6" t="s">
+      <c r="A54" s="5" t="s">
         <v>2050</v>
       </c>
-      <c r="B54" s="6" t="s">
+      <c r="B54" s="5" t="s">
         <v>1901</v>
       </c>
-      <c r="C54" s="6" t="b">
-        <v>1</v>
-      </c>
-      <c r="D54" s="6">
+      <c r="C54" s="5" t="b">
+        <v>1</v>
+      </c>
+      <c r="D54" s="5">
         <v>99</v>
       </c>
-      <c r="E54" s="6" t="s">
+      <c r="E54" s="5" t="s">
         <v>350</v>
       </c>
-      <c r="F54" s="6" t="s">
+      <c r="F54" s="5" t="s">
         <v>350</v>
       </c>
-      <c r="G54" s="6" t="s">
+      <c r="G54" s="5" t="s">
         <v>763</v>
       </c>
-      <c r="H54" s="6" t="s">
+      <c r="H54" s="5" t="s">
         <v>2057</v>
       </c>
-      <c r="I54" s="6">
+      <c r="I54" s="5">
         <v>7500000</v>
       </c>
-      <c r="J54" s="6" t="s">
+      <c r="J54" s="5" t="s">
         <v>2051</v>
       </c>
-      <c r="K54" s="6">
-        <v>1</v>
-      </c>
-      <c r="L54" s="6" t="s">
+      <c r="K54" s="5">
+        <v>1</v>
+      </c>
+      <c r="L54" s="5" t="s">
         <v>350</v>
       </c>
-      <c r="M54" s="6">
+      <c r="M54" s="5">
         <v>99</v>
       </c>
-      <c r="N54" s="6" t="b">
+      <c r="N54" s="5" t="b">
         <v>0</v>
       </c>
-      <c r="O54" s="6" t="s">
+      <c r="O54" s="5" t="s">
         <v>2053</v>
       </c>
     </row>
@@ -26390,35 +26398,35 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:10" s="10" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="10" t="s">
+    <row r="2" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A2" s="9" t="s">
         <v>505</v>
       </c>
-      <c r="B2" s="10">
+      <c r="B2" s="9">
         <v>-140</v>
       </c>
-      <c r="C2" s="10" t="s">
+      <c r="C2" s="9" t="s">
         <v>593</v>
       </c>
-      <c r="D2" s="10">
-        <v>1</v>
-      </c>
-      <c r="E2" s="10" t="s">
+      <c r="D2" s="9">
+        <v>1</v>
+      </c>
+      <c r="E2" s="9" t="s">
         <v>886</v>
       </c>
-      <c r="F2" s="10" t="s">
+      <c r="F2" s="9" t="s">
         <v>890</v>
       </c>
-      <c r="G2" s="10">
+      <c r="G2" s="9">
         <v>0</v>
       </c>
-      <c r="H2" s="10" t="s">
+      <c r="H2" s="9" t="s">
         <v>895</v>
       </c>
-      <c r="I2" s="10" t="s">
+      <c r="I2" s="9" t="s">
         <v>431</v>
       </c>
-      <c r="J2" s="10" t="s">
+      <c r="J2" s="9" t="s">
         <v>351</v>
       </c>
     </row>
@@ -26454,35 +26462,35 @@
         <v>351</v>
       </c>
     </row>
-    <row r="4" spans="1:10" s="10" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="10" t="s">
+    <row r="4" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A4" s="9" t="s">
         <v>512</v>
       </c>
-      <c r="B4" s="10">
+      <c r="B4" s="9">
         <v>-140</v>
       </c>
-      <c r="C4" s="10" t="s">
+      <c r="C4" s="9" t="s">
         <v>593</v>
       </c>
-      <c r="D4" s="10">
-        <v>1</v>
-      </c>
-      <c r="E4" s="10" t="s">
+      <c r="D4" s="9">
+        <v>1</v>
+      </c>
+      <c r="E4" s="9" t="s">
         <v>888</v>
       </c>
-      <c r="F4" s="10" t="s">
+      <c r="F4" s="9" t="s">
         <v>892</v>
       </c>
-      <c r="G4" s="10">
+      <c r="G4" s="9">
         <v>0</v>
       </c>
-      <c r="H4" s="10" t="s">
+      <c r="H4" s="9" t="s">
         <v>2059</v>
       </c>
-      <c r="I4" s="10" t="s">
+      <c r="I4" s="9" t="s">
         <v>431</v>
       </c>
-      <c r="J4" s="10" t="s">
+      <c r="J4" s="9" t="s">
         <v>351</v>
       </c>
     </row>

</xml_diff>